<commit_message>
fix: corregir posiciones de cantidad y talla
</commit_message>
<xml_diff>
--- a/public/PADRON_UNICO_CARGA_MASIVA_FORGE.xlsx
+++ b/public/PADRON_UNICO_CARGA_MASIVA_FORGE.xlsx
@@ -402,8 +402,8 @@
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -430,12 +430,12 @@
       </c>
       <c r="E1" s="5" t="inlineStr">
         <is>
-          <t>TALLA</t>
+          <t>CANTIDAD</t>
         </is>
       </c>
       <c r="F1" s="5" t="inlineStr">
         <is>
-          <t>CANTIDAD</t>
+          <t>TALLA</t>
         </is>
       </c>
       <c r="G1" s="5" t="inlineStr">
@@ -449,8 +449,8 @@
       <c r="B2" s="12" t="str"/>
       <c r="C2" s="13" t="str"/>
       <c r="D2" s="12" t="str"/>
-      <c r="E2" s="12" t="str"/>
-      <c r="F2" s="14" t="str"/>
+      <c r="E2" s="14" t="str"/>
+      <c r="F2" s="12" t="str"/>
       <c r="G2" s="15" t="str"/>
     </row>
     <row r="3">
@@ -458,8 +458,8 @@
       <c r="B3" s="12" t="str"/>
       <c r="C3" s="13" t="str"/>
       <c r="D3" s="12" t="str"/>
-      <c r="E3" s="12" t="str"/>
-      <c r="F3" s="14" t="str"/>
+      <c r="E3" s="14" t="str"/>
+      <c r="F3" s="12" t="str"/>
       <c r="G3" s="15" t="str"/>
     </row>
     <row r="4">
@@ -467,8 +467,8 @@
       <c r="B4" s="12" t="str"/>
       <c r="C4" s="13" t="str"/>
       <c r="D4" s="12" t="str"/>
-      <c r="E4" s="12" t="str"/>
-      <c r="F4" s="14" t="str"/>
+      <c r="E4" s="14" t="str"/>
+      <c r="F4" s="12" t="str"/>
       <c r="G4" s="15" t="str"/>
     </row>
     <row r="5">
@@ -476,8 +476,8 @@
       <c r="B5" s="12" t="str"/>
       <c r="C5" s="13" t="str"/>
       <c r="D5" s="12" t="str"/>
-      <c r="E5" s="12" t="str"/>
-      <c r="F5" s="14" t="str"/>
+      <c r="E5" s="14" t="str"/>
+      <c r="F5" s="12" t="str"/>
       <c r="G5" s="15" t="str"/>
     </row>
     <row r="6">
@@ -485,8 +485,8 @@
       <c r="B6" s="12" t="str"/>
       <c r="C6" s="13" t="str"/>
       <c r="D6" s="12" t="str"/>
-      <c r="E6" s="12" t="str"/>
-      <c r="F6" s="14" t="str"/>
+      <c r="E6" s="14" t="str"/>
+      <c r="F6" s="12" t="str"/>
       <c r="G6" s="15" t="str"/>
     </row>
     <row r="7">
@@ -494,8 +494,8 @@
       <c r="B7" s="12" t="str"/>
       <c r="C7" s="13" t="str"/>
       <c r="D7" s="12" t="str"/>
-      <c r="E7" s="12" t="str"/>
-      <c r="F7" s="14" t="str"/>
+      <c r="E7" s="14" t="str"/>
+      <c r="F7" s="12" t="str"/>
       <c r="G7" s="15" t="str"/>
     </row>
     <row r="8">
@@ -503,8 +503,8 @@
       <c r="B8" s="12" t="str"/>
       <c r="C8" s="13" t="str"/>
       <c r="D8" s="12" t="str"/>
-      <c r="E8" s="12" t="str"/>
-      <c r="F8" s="14" t="str"/>
+      <c r="E8" s="14" t="str"/>
+      <c r="F8" s="12" t="str"/>
       <c r="G8" s="15" t="str"/>
     </row>
     <row r="9">
@@ -512,8 +512,8 @@
       <c r="B9" s="12" t="str"/>
       <c r="C9" s="13" t="str"/>
       <c r="D9" s="12" t="str"/>
-      <c r="E9" s="12" t="str"/>
-      <c r="F9" s="14" t="str"/>
+      <c r="E9" s="14" t="str"/>
+      <c r="F9" s="12" t="str"/>
       <c r="G9" s="15" t="str"/>
     </row>
     <row r="10">
@@ -521,8 +521,8 @@
       <c r="B10" s="12" t="str"/>
       <c r="C10" s="13" t="str"/>
       <c r="D10" s="12" t="str"/>
-      <c r="E10" s="12" t="str"/>
-      <c r="F10" s="14" t="str"/>
+      <c r="E10" s="14" t="str"/>
+      <c r="F10" s="12" t="str"/>
       <c r="G10" s="15" t="str"/>
     </row>
     <row r="11">
@@ -530,8 +530,8 @@
       <c r="B11" s="12" t="str"/>
       <c r="C11" s="13" t="str"/>
       <c r="D11" s="12" t="str"/>
-      <c r="E11" s="12" t="str"/>
-      <c r="F11" s="14" t="str"/>
+      <c r="E11" s="14" t="str"/>
+      <c r="F11" s="12" t="str"/>
       <c r="G11" s="15" t="str"/>
     </row>
     <row r="12">
@@ -539,8 +539,8 @@
       <c r="B12" s="12" t="str"/>
       <c r="C12" s="13" t="str"/>
       <c r="D12" s="12" t="str"/>
-      <c r="E12" s="12" t="str"/>
-      <c r="F12" s="14" t="str"/>
+      <c r="E12" s="14" t="str"/>
+      <c r="F12" s="12" t="str"/>
       <c r="G12" s="15" t="str"/>
     </row>
     <row r="13">
@@ -548,8 +548,8 @@
       <c r="B13" s="12" t="str"/>
       <c r="C13" s="13" t="str"/>
       <c r="D13" s="12" t="str"/>
-      <c r="E13" s="12" t="str"/>
-      <c r="F13" s="14" t="str"/>
+      <c r="E13" s="14" t="str"/>
+      <c r="F13" s="12" t="str"/>
       <c r="G13" s="15" t="str"/>
     </row>
     <row r="14">
@@ -557,8 +557,8 @@
       <c r="B14" s="12" t="str"/>
       <c r="C14" s="13" t="str"/>
       <c r="D14" s="12" t="str"/>
-      <c r="E14" s="12" t="str"/>
-      <c r="F14" s="14" t="str"/>
+      <c r="E14" s="14" t="str"/>
+      <c r="F14" s="12" t="str"/>
       <c r="G14" s="15" t="str"/>
     </row>
     <row r="15">
@@ -566,8 +566,8 @@
       <c r="B15" s="12" t="str"/>
       <c r="C15" s="13" t="str"/>
       <c r="D15" s="12" t="str"/>
-      <c r="E15" s="12" t="str"/>
-      <c r="F15" s="14" t="str"/>
+      <c r="E15" s="14" t="str"/>
+      <c r="F15" s="12" t="str"/>
       <c r="G15" s="15" t="str"/>
     </row>
     <row r="16">
@@ -575,8 +575,8 @@
       <c r="B16" s="12" t="str"/>
       <c r="C16" s="13" t="str"/>
       <c r="D16" s="12" t="str"/>
-      <c r="E16" s="12" t="str"/>
-      <c r="F16" s="14" t="str"/>
+      <c r="E16" s="14" t="str"/>
+      <c r="F16" s="12" t="str"/>
       <c r="G16" s="15" t="str"/>
     </row>
     <row r="17">
@@ -584,8 +584,8 @@
       <c r="B17" s="12" t="str"/>
       <c r="C17" s="13" t="str"/>
       <c r="D17" s="12" t="str"/>
-      <c r="E17" s="12" t="str"/>
-      <c r="F17" s="14" t="str"/>
+      <c r="E17" s="14" t="str"/>
+      <c r="F17" s="12" t="str"/>
       <c r="G17" s="15" t="str"/>
     </row>
     <row r="18">
@@ -593,8 +593,8 @@
       <c r="B18" s="12" t="str"/>
       <c r="C18" s="13" t="str"/>
       <c r="D18" s="12" t="str"/>
-      <c r="E18" s="12" t="str"/>
-      <c r="F18" s="14" t="str"/>
+      <c r="E18" s="14" t="str"/>
+      <c r="F18" s="12" t="str"/>
       <c r="G18" s="15" t="str"/>
     </row>
     <row r="19">
@@ -602,8 +602,8 @@
       <c r="B19" s="12" t="str"/>
       <c r="C19" s="13" t="str"/>
       <c r="D19" s="12" t="str"/>
-      <c r="E19" s="12" t="str"/>
-      <c r="F19" s="14" t="str"/>
+      <c r="E19" s="14" t="str"/>
+      <c r="F19" s="12" t="str"/>
       <c r="G19" s="15" t="str"/>
     </row>
     <row r="20">
@@ -611,8 +611,8 @@
       <c r="B20" s="12" t="str"/>
       <c r="C20" s="13" t="str"/>
       <c r="D20" s="12" t="str"/>
-      <c r="E20" s="12" t="str"/>
-      <c r="F20" s="14" t="str"/>
+      <c r="E20" s="14" t="str"/>
+      <c r="F20" s="12" t="str"/>
       <c r="G20" s="15" t="str"/>
     </row>
     <row r="21">
@@ -620,8 +620,8 @@
       <c r="B21" s="12" t="str"/>
       <c r="C21" s="13" t="str"/>
       <c r="D21" s="12" t="str"/>
-      <c r="E21" s="12" t="str"/>
-      <c r="F21" s="14" t="str"/>
+      <c r="E21" s="14" t="str"/>
+      <c r="F21" s="12" t="str"/>
       <c r="G21" s="15" t="str"/>
     </row>
     <row r="22">
@@ -629,8 +629,8 @@
       <c r="B22" s="12" t="str"/>
       <c r="C22" s="13" t="str"/>
       <c r="D22" s="12" t="str"/>
-      <c r="E22" s="12" t="str"/>
-      <c r="F22" s="14" t="str"/>
+      <c r="E22" s="14" t="str"/>
+      <c r="F22" s="12" t="str"/>
       <c r="G22" s="15" t="str"/>
     </row>
     <row r="23">
@@ -638,8 +638,8 @@
       <c r="B23" s="12" t="str"/>
       <c r="C23" s="13" t="str"/>
       <c r="D23" s="12" t="str"/>
-      <c r="E23" s="12" t="str"/>
-      <c r="F23" s="14" t="str"/>
+      <c r="E23" s="14" t="str"/>
+      <c r="F23" s="12" t="str"/>
       <c r="G23" s="15" t="str"/>
     </row>
     <row r="24">
@@ -647,8 +647,8 @@
       <c r="B24" s="12" t="str"/>
       <c r="C24" s="13" t="str"/>
       <c r="D24" s="12" t="str"/>
-      <c r="E24" s="12" t="str"/>
-      <c r="F24" s="14" t="str"/>
+      <c r="E24" s="14" t="str"/>
+      <c r="F24" s="12" t="str"/>
       <c r="G24" s="15" t="str"/>
     </row>
     <row r="25">
@@ -656,8 +656,8 @@
       <c r="B25" s="12" t="str"/>
       <c r="C25" s="13" t="str"/>
       <c r="D25" s="12" t="str"/>
-      <c r="E25" s="12" t="str"/>
-      <c r="F25" s="14" t="str"/>
+      <c r="E25" s="14" t="str"/>
+      <c r="F25" s="12" t="str"/>
       <c r="G25" s="15" t="str"/>
     </row>
     <row r="26">
@@ -665,8 +665,8 @@
       <c r="B26" s="12" t="str"/>
       <c r="C26" s="13" t="str"/>
       <c r="D26" s="12" t="str"/>
-      <c r="E26" s="12" t="str"/>
-      <c r="F26" s="14" t="str"/>
+      <c r="E26" s="14" t="str"/>
+      <c r="F26" s="12" t="str"/>
       <c r="G26" s="15" t="str"/>
     </row>
     <row r="27">
@@ -674,8 +674,8 @@
       <c r="B27" s="12" t="str"/>
       <c r="C27" s="13" t="str"/>
       <c r="D27" s="12" t="str"/>
-      <c r="E27" s="12" t="str"/>
-      <c r="F27" s="14" t="str"/>
+      <c r="E27" s="14" t="str"/>
+      <c r="F27" s="12" t="str"/>
       <c r="G27" s="15" t="str"/>
     </row>
     <row r="28">
@@ -683,8 +683,8 @@
       <c r="B28" s="12" t="str"/>
       <c r="C28" s="13" t="str"/>
       <c r="D28" s="12" t="str"/>
-      <c r="E28" s="12" t="str"/>
-      <c r="F28" s="14" t="str"/>
+      <c r="E28" s="14" t="str"/>
+      <c r="F28" s="12" t="str"/>
       <c r="G28" s="15" t="str"/>
     </row>
     <row r="29">
@@ -692,8 +692,8 @@
       <c r="B29" s="12" t="str"/>
       <c r="C29" s="13" t="str"/>
       <c r="D29" s="12" t="str"/>
-      <c r="E29" s="12" t="str"/>
-      <c r="F29" s="14" t="str"/>
+      <c r="E29" s="14" t="str"/>
+      <c r="F29" s="12" t="str"/>
       <c r="G29" s="15" t="str"/>
     </row>
     <row r="30">
@@ -701,8 +701,8 @@
       <c r="B30" s="12" t="str"/>
       <c r="C30" s="13" t="str"/>
       <c r="D30" s="12" t="str"/>
-      <c r="E30" s="12" t="str"/>
-      <c r="F30" s="14" t="str"/>
+      <c r="E30" s="14" t="str"/>
+      <c r="F30" s="12" t="str"/>
       <c r="G30" s="15" t="str"/>
     </row>
     <row r="31">
@@ -710,8 +710,8 @@
       <c r="B31" s="12" t="str"/>
       <c r="C31" s="13" t="str"/>
       <c r="D31" s="12" t="str"/>
-      <c r="E31" s="12" t="str"/>
-      <c r="F31" s="14" t="str"/>
+      <c r="E31" s="14" t="str"/>
+      <c r="F31" s="12" t="str"/>
       <c r="G31" s="15" t="str"/>
     </row>
     <row r="32">
@@ -719,8 +719,8 @@
       <c r="B32" s="12" t="str"/>
       <c r="C32" s="13" t="str"/>
       <c r="D32" s="12" t="str"/>
-      <c r="E32" s="12" t="str"/>
-      <c r="F32" s="14" t="str"/>
+      <c r="E32" s="14" t="str"/>
+      <c r="F32" s="12" t="str"/>
       <c r="G32" s="15" t="str"/>
     </row>
     <row r="33">
@@ -728,8 +728,8 @@
       <c r="B33" s="12" t="str"/>
       <c r="C33" s="13" t="str"/>
       <c r="D33" s="12" t="str"/>
-      <c r="E33" s="12" t="str"/>
-      <c r="F33" s="14" t="str"/>
+      <c r="E33" s="14" t="str"/>
+      <c r="F33" s="12" t="str"/>
       <c r="G33" s="15" t="str"/>
     </row>
     <row r="34">
@@ -737,8 +737,8 @@
       <c r="B34" s="12" t="str"/>
       <c r="C34" s="13" t="str"/>
       <c r="D34" s="12" t="str"/>
-      <c r="E34" s="12" t="str"/>
-      <c r="F34" s="14" t="str"/>
+      <c r="E34" s="14" t="str"/>
+      <c r="F34" s="12" t="str"/>
       <c r="G34" s="15" t="str"/>
     </row>
     <row r="35">
@@ -746,8 +746,8 @@
       <c r="B35" s="12" t="str"/>
       <c r="C35" s="13" t="str"/>
       <c r="D35" s="12" t="str"/>
-      <c r="E35" s="12" t="str"/>
-      <c r="F35" s="14" t="str"/>
+      <c r="E35" s="14" t="str"/>
+      <c r="F35" s="12" t="str"/>
       <c r="G35" s="15" t="str"/>
     </row>
     <row r="36">
@@ -755,8 +755,8 @@
       <c r="B36" s="12" t="str"/>
       <c r="C36" s="13" t="str"/>
       <c r="D36" s="12" t="str"/>
-      <c r="E36" s="12" t="str"/>
-      <c r="F36" s="14" t="str"/>
+      <c r="E36" s="14" t="str"/>
+      <c r="F36" s="12" t="str"/>
       <c r="G36" s="15" t="str"/>
     </row>
     <row r="37">
@@ -764,8 +764,8 @@
       <c r="B37" s="12" t="str"/>
       <c r="C37" s="13" t="str"/>
       <c r="D37" s="12" t="str"/>
-      <c r="E37" s="12" t="str"/>
-      <c r="F37" s="14" t="str"/>
+      <c r="E37" s="14" t="str"/>
+      <c r="F37" s="12" t="str"/>
       <c r="G37" s="15" t="str"/>
     </row>
     <row r="38">
@@ -773,8 +773,8 @@
       <c r="B38" s="12" t="str"/>
       <c r="C38" s="13" t="str"/>
       <c r="D38" s="12" t="str"/>
-      <c r="E38" s="12" t="str"/>
-      <c r="F38" s="14" t="str"/>
+      <c r="E38" s="14" t="str"/>
+      <c r="F38" s="12" t="str"/>
       <c r="G38" s="15" t="str"/>
     </row>
     <row r="39">
@@ -782,8 +782,8 @@
       <c r="B39" s="12" t="str"/>
       <c r="C39" s="13" t="str"/>
       <c r="D39" s="12" t="str"/>
-      <c r="E39" s="12" t="str"/>
-      <c r="F39" s="14" t="str"/>
+      <c r="E39" s="14" t="str"/>
+      <c r="F39" s="12" t="str"/>
       <c r="G39" s="15" t="str"/>
     </row>
     <row r="40">
@@ -791,8 +791,8 @@
       <c r="B40" s="12" t="str"/>
       <c r="C40" s="13" t="str"/>
       <c r="D40" s="12" t="str"/>
-      <c r="E40" s="12" t="str"/>
-      <c r="F40" s="14" t="str"/>
+      <c r="E40" s="14" t="str"/>
+      <c r="F40" s="12" t="str"/>
       <c r="G40" s="15" t="str"/>
     </row>
     <row r="41">
@@ -800,8 +800,8 @@
       <c r="B41" s="12" t="str"/>
       <c r="C41" s="13" t="str"/>
       <c r="D41" s="12" t="str"/>
-      <c r="E41" s="12" t="str"/>
-      <c r="F41" s="14" t="str"/>
+      <c r="E41" s="14" t="str"/>
+      <c r="F41" s="12" t="str"/>
       <c r="G41" s="15" t="str"/>
     </row>
     <row r="42">
@@ -809,8 +809,8 @@
       <c r="B42" s="12" t="str"/>
       <c r="C42" s="13" t="str"/>
       <c r="D42" s="12" t="str"/>
-      <c r="E42" s="12" t="str"/>
-      <c r="F42" s="14" t="str"/>
+      <c r="E42" s="14" t="str"/>
+      <c r="F42" s="12" t="str"/>
       <c r="G42" s="15" t="str"/>
     </row>
     <row r="43">
@@ -818,8 +818,8 @@
       <c r="B43" s="12" t="str"/>
       <c r="C43" s="13" t="str"/>
       <c r="D43" s="12" t="str"/>
-      <c r="E43" s="12" t="str"/>
-      <c r="F43" s="14" t="str"/>
+      <c r="E43" s="14" t="str"/>
+      <c r="F43" s="12" t="str"/>
       <c r="G43" s="15" t="str"/>
     </row>
     <row r="44">
@@ -827,8 +827,8 @@
       <c r="B44" s="12" t="str"/>
       <c r="C44" s="13" t="str"/>
       <c r="D44" s="12" t="str"/>
-      <c r="E44" s="12" t="str"/>
-      <c r="F44" s="14" t="str"/>
+      <c r="E44" s="14" t="str"/>
+      <c r="F44" s="12" t="str"/>
       <c r="G44" s="15" t="str"/>
     </row>
     <row r="45">
@@ -836,8 +836,8 @@
       <c r="B45" s="12" t="str"/>
       <c r="C45" s="13" t="str"/>
       <c r="D45" s="12" t="str"/>
-      <c r="E45" s="12" t="str"/>
-      <c r="F45" s="14" t="str"/>
+      <c r="E45" s="14" t="str"/>
+      <c r="F45" s="12" t="str"/>
       <c r="G45" s="15" t="str"/>
     </row>
     <row r="46">
@@ -845,8 +845,8 @@
       <c r="B46" s="12" t="str"/>
       <c r="C46" s="13" t="str"/>
       <c r="D46" s="12" t="str"/>
-      <c r="E46" s="12" t="str"/>
-      <c r="F46" s="14" t="str"/>
+      <c r="E46" s="14" t="str"/>
+      <c r="F46" s="12" t="str"/>
       <c r="G46" s="15" t="str"/>
     </row>
     <row r="47">
@@ -854,8 +854,8 @@
       <c r="B47" s="12" t="str"/>
       <c r="C47" s="13" t="str"/>
       <c r="D47" s="12" t="str"/>
-      <c r="E47" s="12" t="str"/>
-      <c r="F47" s="14" t="str"/>
+      <c r="E47" s="14" t="str"/>
+      <c r="F47" s="12" t="str"/>
       <c r="G47" s="15" t="str"/>
     </row>
     <row r="48">
@@ -863,8 +863,8 @@
       <c r="B48" s="12" t="str"/>
       <c r="C48" s="13" t="str"/>
       <c r="D48" s="12" t="str"/>
-      <c r="E48" s="12" t="str"/>
-      <c r="F48" s="14" t="str"/>
+      <c r="E48" s="14" t="str"/>
+      <c r="F48" s="12" t="str"/>
       <c r="G48" s="15" t="str"/>
     </row>
     <row r="49">
@@ -872,8 +872,8 @@
       <c r="B49" s="12" t="str"/>
       <c r="C49" s="13" t="str"/>
       <c r="D49" s="12" t="str"/>
-      <c r="E49" s="12" t="str"/>
-      <c r="F49" s="14" t="str"/>
+      <c r="E49" s="14" t="str"/>
+      <c r="F49" s="12" t="str"/>
       <c r="G49" s="15" t="str"/>
     </row>
     <row r="50">
@@ -881,8 +881,8 @@
       <c r="B50" s="12" t="str"/>
       <c r="C50" s="13" t="str"/>
       <c r="D50" s="12" t="str"/>
-      <c r="E50" s="12" t="str"/>
-      <c r="F50" s="14" t="str"/>
+      <c r="E50" s="14" t="str"/>
+      <c r="F50" s="12" t="str"/>
       <c r="G50" s="15" t="str"/>
     </row>
     <row r="51">
@@ -890,8 +890,8 @@
       <c r="B51" s="12" t="str"/>
       <c r="C51" s="13" t="str"/>
       <c r="D51" s="12" t="str"/>
-      <c r="E51" s="12" t="str"/>
-      <c r="F51" s="14" t="str"/>
+      <c r="E51" s="14" t="str"/>
+      <c r="F51" s="12" t="str"/>
       <c r="G51" s="15" t="str"/>
     </row>
     <row r="52">
@@ -899,8 +899,8 @@
       <c r="B52" s="12" t="str"/>
       <c r="C52" s="13" t="str"/>
       <c r="D52" s="12" t="str"/>
-      <c r="E52" s="12" t="str"/>
-      <c r="F52" s="14" t="str"/>
+      <c r="E52" s="14" t="str"/>
+      <c r="F52" s="12" t="str"/>
       <c r="G52" s="15" t="str"/>
     </row>
     <row r="53">
@@ -908,8 +908,8 @@
       <c r="B53" s="12" t="str"/>
       <c r="C53" s="13" t="str"/>
       <c r="D53" s="12" t="str"/>
-      <c r="E53" s="12" t="str"/>
-      <c r="F53" s="14" t="str"/>
+      <c r="E53" s="14" t="str"/>
+      <c r="F53" s="12" t="str"/>
       <c r="G53" s="15" t="str"/>
     </row>
     <row r="54">
@@ -917,8 +917,8 @@
       <c r="B54" s="12" t="str"/>
       <c r="C54" s="13" t="str"/>
       <c r="D54" s="12" t="str"/>
-      <c r="E54" s="12" t="str"/>
-      <c r="F54" s="14" t="str"/>
+      <c r="E54" s="14" t="str"/>
+      <c r="F54" s="12" t="str"/>
       <c r="G54" s="15" t="str"/>
     </row>
     <row r="55">
@@ -926,8 +926,8 @@
       <c r="B55" s="12" t="str"/>
       <c r="C55" s="13" t="str"/>
       <c r="D55" s="12" t="str"/>
-      <c r="E55" s="12" t="str"/>
-      <c r="F55" s="14" t="str"/>
+      <c r="E55" s="14" t="str"/>
+      <c r="F55" s="12" t="str"/>
       <c r="G55" s="15" t="str"/>
     </row>
     <row r="56">
@@ -935,8 +935,8 @@
       <c r="B56" s="12" t="str"/>
       <c r="C56" s="13" t="str"/>
       <c r="D56" s="12" t="str"/>
-      <c r="E56" s="12" t="str"/>
-      <c r="F56" s="14" t="str"/>
+      <c r="E56" s="14" t="str"/>
+      <c r="F56" s="12" t="str"/>
       <c r="G56" s="15" t="str"/>
     </row>
     <row r="57">
@@ -944,8 +944,8 @@
       <c r="B57" s="12" t="str"/>
       <c r="C57" s="13" t="str"/>
       <c r="D57" s="12" t="str"/>
-      <c r="E57" s="12" t="str"/>
-      <c r="F57" s="14" t="str"/>
+      <c r="E57" s="14" t="str"/>
+      <c r="F57" s="12" t="str"/>
       <c r="G57" s="15" t="str"/>
     </row>
     <row r="58">
@@ -953,8 +953,8 @@
       <c r="B58" s="12" t="str"/>
       <c r="C58" s="13" t="str"/>
       <c r="D58" s="12" t="str"/>
-      <c r="E58" s="12" t="str"/>
-      <c r="F58" s="14" t="str"/>
+      <c r="E58" s="14" t="str"/>
+      <c r="F58" s="12" t="str"/>
       <c r="G58" s="15" t="str"/>
     </row>
     <row r="59">
@@ -962,8 +962,8 @@
       <c r="B59" s="12" t="str"/>
       <c r="C59" s="13" t="str"/>
       <c r="D59" s="12" t="str"/>
-      <c r="E59" s="12" t="str"/>
-      <c r="F59" s="14" t="str"/>
+      <c r="E59" s="14" t="str"/>
+      <c r="F59" s="12" t="str"/>
       <c r="G59" s="15" t="str"/>
     </row>
     <row r="60">
@@ -971,8 +971,8 @@
       <c r="B60" s="12" t="str"/>
       <c r="C60" s="13" t="str"/>
       <c r="D60" s="12" t="str"/>
-      <c r="E60" s="12" t="str"/>
-      <c r="F60" s="14" t="str"/>
+      <c r="E60" s="14" t="str"/>
+      <c r="F60" s="12" t="str"/>
       <c r="G60" s="15" t="str"/>
     </row>
     <row r="61">
@@ -980,8 +980,8 @@
       <c r="B61" s="12" t="str"/>
       <c r="C61" s="13" t="str"/>
       <c r="D61" s="12" t="str"/>
-      <c r="E61" s="12" t="str"/>
-      <c r="F61" s="14" t="str"/>
+      <c r="E61" s="14" t="str"/>
+      <c r="F61" s="12" t="str"/>
       <c r="G61" s="15" t="str"/>
     </row>
     <row r="62">
@@ -989,8 +989,8 @@
       <c r="B62" s="12" t="str"/>
       <c r="C62" s="13" t="str"/>
       <c r="D62" s="12" t="str"/>
-      <c r="E62" s="12" t="str"/>
-      <c r="F62" s="14" t="str"/>
+      <c r="E62" s="14" t="str"/>
+      <c r="F62" s="12" t="str"/>
       <c r="G62" s="15" t="str"/>
     </row>
     <row r="63">
@@ -998,8 +998,8 @@
       <c r="B63" s="12" t="str"/>
       <c r="C63" s="13" t="str"/>
       <c r="D63" s="12" t="str"/>
-      <c r="E63" s="12" t="str"/>
-      <c r="F63" s="14" t="str"/>
+      <c r="E63" s="14" t="str"/>
+      <c r="F63" s="12" t="str"/>
       <c r="G63" s="15" t="str"/>
     </row>
     <row r="64">
@@ -1007,8 +1007,8 @@
       <c r="B64" s="12" t="str"/>
       <c r="C64" s="13" t="str"/>
       <c r="D64" s="12" t="str"/>
-      <c r="E64" s="12" t="str"/>
-      <c r="F64" s="14" t="str"/>
+      <c r="E64" s="14" t="str"/>
+      <c r="F64" s="12" t="str"/>
       <c r="G64" s="15" t="str"/>
     </row>
     <row r="65">
@@ -1016,8 +1016,8 @@
       <c r="B65" s="12" t="str"/>
       <c r="C65" s="13" t="str"/>
       <c r="D65" s="12" t="str"/>
-      <c r="E65" s="12" t="str"/>
-      <c r="F65" s="14" t="str"/>
+      <c r="E65" s="14" t="str"/>
+      <c r="F65" s="12" t="str"/>
       <c r="G65" s="15" t="str"/>
     </row>
     <row r="66">
@@ -1025,8 +1025,8 @@
       <c r="B66" s="12" t="str"/>
       <c r="C66" s="13" t="str"/>
       <c r="D66" s="12" t="str"/>
-      <c r="E66" s="12" t="str"/>
-      <c r="F66" s="14" t="str"/>
+      <c r="E66" s="14" t="str"/>
+      <c r="F66" s="12" t="str"/>
       <c r="G66" s="15" t="str"/>
     </row>
     <row r="67">
@@ -1034,8 +1034,8 @@
       <c r="B67" s="12" t="str"/>
       <c r="C67" s="13" t="str"/>
       <c r="D67" s="12" t="str"/>
-      <c r="E67" s="12" t="str"/>
-      <c r="F67" s="14" t="str"/>
+      <c r="E67" s="14" t="str"/>
+      <c r="F67" s="12" t="str"/>
       <c r="G67" s="15" t="str"/>
     </row>
     <row r="68">
@@ -1043,8 +1043,8 @@
       <c r="B68" s="12" t="str"/>
       <c r="C68" s="13" t="str"/>
       <c r="D68" s="12" t="str"/>
-      <c r="E68" s="12" t="str"/>
-      <c r="F68" s="14" t="str"/>
+      <c r="E68" s="14" t="str"/>
+      <c r="F68" s="12" t="str"/>
       <c r="G68" s="15" t="str"/>
     </row>
     <row r="69">
@@ -1052,8 +1052,8 @@
       <c r="B69" s="12" t="str"/>
       <c r="C69" s="13" t="str"/>
       <c r="D69" s="12" t="str"/>
-      <c r="E69" s="12" t="str"/>
-      <c r="F69" s="14" t="str"/>
+      <c r="E69" s="14" t="str"/>
+      <c r="F69" s="12" t="str"/>
       <c r="G69" s="15" t="str"/>
     </row>
     <row r="70">
@@ -1061,8 +1061,8 @@
       <c r="B70" s="12" t="str"/>
       <c r="C70" s="13" t="str"/>
       <c r="D70" s="12" t="str"/>
-      <c r="E70" s="12" t="str"/>
-      <c r="F70" s="14" t="str"/>
+      <c r="E70" s="14" t="str"/>
+      <c r="F70" s="12" t="str"/>
       <c r="G70" s="15" t="str"/>
     </row>
     <row r="71">
@@ -1070,8 +1070,8 @@
       <c r="B71" s="12" t="str"/>
       <c r="C71" s="13" t="str"/>
       <c r="D71" s="12" t="str"/>
-      <c r="E71" s="12" t="str"/>
-      <c r="F71" s="14" t="str"/>
+      <c r="E71" s="14" t="str"/>
+      <c r="F71" s="12" t="str"/>
       <c r="G71" s="15" t="str"/>
     </row>
     <row r="72">
@@ -1079,8 +1079,8 @@
       <c r="B72" s="12" t="str"/>
       <c r="C72" s="13" t="str"/>
       <c r="D72" s="12" t="str"/>
-      <c r="E72" s="12" t="str"/>
-      <c r="F72" s="14" t="str"/>
+      <c r="E72" s="14" t="str"/>
+      <c r="F72" s="12" t="str"/>
       <c r="G72" s="15" t="str"/>
     </row>
     <row r="73">
@@ -1088,8 +1088,8 @@
       <c r="B73" s="12" t="str"/>
       <c r="C73" s="13" t="str"/>
       <c r="D73" s="12" t="str"/>
-      <c r="E73" s="12" t="str"/>
-      <c r="F73" s="14" t="str"/>
+      <c r="E73" s="14" t="str"/>
+      <c r="F73" s="12" t="str"/>
       <c r="G73" s="15" t="str"/>
     </row>
     <row r="74">
@@ -1097,8 +1097,8 @@
       <c r="B74" s="12" t="str"/>
       <c r="C74" s="13" t="str"/>
       <c r="D74" s="12" t="str"/>
-      <c r="E74" s="12" t="str"/>
-      <c r="F74" s="14" t="str"/>
+      <c r="E74" s="14" t="str"/>
+      <c r="F74" s="12" t="str"/>
       <c r="G74" s="15" t="str"/>
     </row>
     <row r="75">
@@ -1106,8 +1106,8 @@
       <c r="B75" s="12" t="str"/>
       <c r="C75" s="13" t="str"/>
       <c r="D75" s="12" t="str"/>
-      <c r="E75" s="12" t="str"/>
-      <c r="F75" s="14" t="str"/>
+      <c r="E75" s="14" t="str"/>
+      <c r="F75" s="12" t="str"/>
       <c r="G75" s="15" t="str"/>
     </row>
     <row r="76">
@@ -1115,8 +1115,8 @@
       <c r="B76" s="12" t="str"/>
       <c r="C76" s="13" t="str"/>
       <c r="D76" s="12" t="str"/>
-      <c r="E76" s="12" t="str"/>
-      <c r="F76" s="14" t="str"/>
+      <c r="E76" s="14" t="str"/>
+      <c r="F76" s="12" t="str"/>
       <c r="G76" s="15" t="str"/>
     </row>
     <row r="77">
@@ -1124,8 +1124,8 @@
       <c r="B77" s="12" t="str"/>
       <c r="C77" s="13" t="str"/>
       <c r="D77" s="12" t="str"/>
-      <c r="E77" s="12" t="str"/>
-      <c r="F77" s="14" t="str"/>
+      <c r="E77" s="14" t="str"/>
+      <c r="F77" s="12" t="str"/>
       <c r="G77" s="15" t="str"/>
     </row>
     <row r="78">
@@ -1133,8 +1133,8 @@
       <c r="B78" s="12" t="str"/>
       <c r="C78" s="13" t="str"/>
       <c r="D78" s="12" t="str"/>
-      <c r="E78" s="12" t="str"/>
-      <c r="F78" s="14" t="str"/>
+      <c r="E78" s="14" t="str"/>
+      <c r="F78" s="12" t="str"/>
       <c r="G78" s="15" t="str"/>
     </row>
     <row r="79">
@@ -1142,8 +1142,8 @@
       <c r="B79" s="12" t="str"/>
       <c r="C79" s="13" t="str"/>
       <c r="D79" s="12" t="str"/>
-      <c r="E79" s="12" t="str"/>
-      <c r="F79" s="14" t="str"/>
+      <c r="E79" s="14" t="str"/>
+      <c r="F79" s="12" t="str"/>
       <c r="G79" s="15" t="str"/>
     </row>
     <row r="80">
@@ -1151,8 +1151,8 @@
       <c r="B80" s="12" t="str"/>
       <c r="C80" s="13" t="str"/>
       <c r="D80" s="12" t="str"/>
-      <c r="E80" s="12" t="str"/>
-      <c r="F80" s="14" t="str"/>
+      <c r="E80" s="14" t="str"/>
+      <c r="F80" s="12" t="str"/>
       <c r="G80" s="15" t="str"/>
     </row>
     <row r="81">
@@ -1160,8 +1160,8 @@
       <c r="B81" s="12" t="str"/>
       <c r="C81" s="13" t="str"/>
       <c r="D81" s="12" t="str"/>
-      <c r="E81" s="12" t="str"/>
-      <c r="F81" s="14" t="str"/>
+      <c r="E81" s="14" t="str"/>
+      <c r="F81" s="12" t="str"/>
       <c r="G81" s="15" t="str"/>
     </row>
     <row r="82">
@@ -1169,8 +1169,8 @@
       <c r="B82" s="12" t="str"/>
       <c r="C82" s="13" t="str"/>
       <c r="D82" s="12" t="str"/>
-      <c r="E82" s="12" t="str"/>
-      <c r="F82" s="14" t="str"/>
+      <c r="E82" s="14" t="str"/>
+      <c r="F82" s="12" t="str"/>
       <c r="G82" s="15" t="str"/>
     </row>
     <row r="83">
@@ -1178,8 +1178,8 @@
       <c r="B83" s="12" t="str"/>
       <c r="C83" s="13" t="str"/>
       <c r="D83" s="12" t="str"/>
-      <c r="E83" s="12" t="str"/>
-      <c r="F83" s="14" t="str"/>
+      <c r="E83" s="14" t="str"/>
+      <c r="F83" s="12" t="str"/>
       <c r="G83" s="15" t="str"/>
     </row>
     <row r="84">
@@ -1187,8 +1187,8 @@
       <c r="B84" s="12" t="str"/>
       <c r="C84" s="13" t="str"/>
       <c r="D84" s="12" t="str"/>
-      <c r="E84" s="12" t="str"/>
-      <c r="F84" s="14" t="str"/>
+      <c r="E84" s="14" t="str"/>
+      <c r="F84" s="12" t="str"/>
       <c r="G84" s="15" t="str"/>
     </row>
     <row r="85">
@@ -1196,8 +1196,8 @@
       <c r="B85" s="12" t="str"/>
       <c r="C85" s="13" t="str"/>
       <c r="D85" s="12" t="str"/>
-      <c r="E85" s="12" t="str"/>
-      <c r="F85" s="14" t="str"/>
+      <c r="E85" s="14" t="str"/>
+      <c r="F85" s="12" t="str"/>
       <c r="G85" s="15" t="str"/>
     </row>
     <row r="86">
@@ -1205,8 +1205,8 @@
       <c r="B86" s="12" t="str"/>
       <c r="C86" s="13" t="str"/>
       <c r="D86" s="12" t="str"/>
-      <c r="E86" s="12" t="str"/>
-      <c r="F86" s="14" t="str"/>
+      <c r="E86" s="14" t="str"/>
+      <c r="F86" s="12" t="str"/>
       <c r="G86" s="15" t="str"/>
     </row>
     <row r="87">
@@ -1214,8 +1214,8 @@
       <c r="B87" s="12" t="str"/>
       <c r="C87" s="13" t="str"/>
       <c r="D87" s="12" t="str"/>
-      <c r="E87" s="12" t="str"/>
-      <c r="F87" s="14" t="str"/>
+      <c r="E87" s="14" t="str"/>
+      <c r="F87" s="12" t="str"/>
       <c r="G87" s="15" t="str"/>
     </row>
     <row r="88">
@@ -1223,8 +1223,8 @@
       <c r="B88" s="12" t="str"/>
       <c r="C88" s="13" t="str"/>
       <c r="D88" s="12" t="str"/>
-      <c r="E88" s="12" t="str"/>
-      <c r="F88" s="14" t="str"/>
+      <c r="E88" s="14" t="str"/>
+      <c r="F88" s="12" t="str"/>
       <c r="G88" s="15" t="str"/>
     </row>
     <row r="89">
@@ -1232,8 +1232,8 @@
       <c r="B89" s="12" t="str"/>
       <c r="C89" s="13" t="str"/>
       <c r="D89" s="12" t="str"/>
-      <c r="E89" s="12" t="str"/>
-      <c r="F89" s="14" t="str"/>
+      <c r="E89" s="14" t="str"/>
+      <c r="F89" s="12" t="str"/>
       <c r="G89" s="15" t="str"/>
     </row>
     <row r="90">
@@ -1241,8 +1241,8 @@
       <c r="B90" s="12" t="str"/>
       <c r="C90" s="13" t="str"/>
       <c r="D90" s="12" t="str"/>
-      <c r="E90" s="12" t="str"/>
-      <c r="F90" s="14" t="str"/>
+      <c r="E90" s="14" t="str"/>
+      <c r="F90" s="12" t="str"/>
       <c r="G90" s="15" t="str"/>
     </row>
     <row r="91">
@@ -1250,8 +1250,8 @@
       <c r="B91" s="12" t="str"/>
       <c r="C91" s="13" t="str"/>
       <c r="D91" s="12" t="str"/>
-      <c r="E91" s="12" t="str"/>
-      <c r="F91" s="14" t="str"/>
+      <c r="E91" s="14" t="str"/>
+      <c r="F91" s="12" t="str"/>
       <c r="G91" s="15" t="str"/>
     </row>
     <row r="92">
@@ -1259,8 +1259,8 @@
       <c r="B92" s="12" t="str"/>
       <c r="C92" s="13" t="str"/>
       <c r="D92" s="12" t="str"/>
-      <c r="E92" s="12" t="str"/>
-      <c r="F92" s="14" t="str"/>
+      <c r="E92" s="14" t="str"/>
+      <c r="F92" s="12" t="str"/>
       <c r="G92" s="15" t="str"/>
     </row>
     <row r="93">
@@ -1268,8 +1268,8 @@
       <c r="B93" s="12" t="str"/>
       <c r="C93" s="13" t="str"/>
       <c r="D93" s="12" t="str"/>
-      <c r="E93" s="12" t="str"/>
-      <c r="F93" s="14" t="str"/>
+      <c r="E93" s="14" t="str"/>
+      <c r="F93" s="12" t="str"/>
       <c r="G93" s="15" t="str"/>
     </row>
     <row r="94">
@@ -1277,8 +1277,8 @@
       <c r="B94" s="12" t="str"/>
       <c r="C94" s="13" t="str"/>
       <c r="D94" s="12" t="str"/>
-      <c r="E94" s="12" t="str"/>
-      <c r="F94" s="14" t="str"/>
+      <c r="E94" s="14" t="str"/>
+      <c r="F94" s="12" t="str"/>
       <c r="G94" s="15" t="str"/>
     </row>
     <row r="95">
@@ -1286,8 +1286,8 @@
       <c r="B95" s="12" t="str"/>
       <c r="C95" s="13" t="str"/>
       <c r="D95" s="12" t="str"/>
-      <c r="E95" s="12" t="str"/>
-      <c r="F95" s="14" t="str"/>
+      <c r="E95" s="14" t="str"/>
+      <c r="F95" s="12" t="str"/>
       <c r="G95" s="15" t="str"/>
     </row>
     <row r="96">
@@ -1295,8 +1295,8 @@
       <c r="B96" s="12" t="str"/>
       <c r="C96" s="13" t="str"/>
       <c r="D96" s="12" t="str"/>
-      <c r="E96" s="12" t="str"/>
-      <c r="F96" s="14" t="str"/>
+      <c r="E96" s="14" t="str"/>
+      <c r="F96" s="12" t="str"/>
       <c r="G96" s="15" t="str"/>
     </row>
     <row r="97">
@@ -1304,8 +1304,8 @@
       <c r="B97" s="12" t="str"/>
       <c r="C97" s="13" t="str"/>
       <c r="D97" s="12" t="str"/>
-      <c r="E97" s="12" t="str"/>
-      <c r="F97" s="14" t="str"/>
+      <c r="E97" s="14" t="str"/>
+      <c r="F97" s="12" t="str"/>
       <c r="G97" s="15" t="str"/>
     </row>
     <row r="98">
@@ -1313,8 +1313,8 @@
       <c r="B98" s="12" t="str"/>
       <c r="C98" s="13" t="str"/>
       <c r="D98" s="12" t="str"/>
-      <c r="E98" s="12" t="str"/>
-      <c r="F98" s="14" t="str"/>
+      <c r="E98" s="14" t="str"/>
+      <c r="F98" s="12" t="str"/>
       <c r="G98" s="15" t="str"/>
     </row>
     <row r="99">
@@ -1322,8 +1322,8 @@
       <c r="B99" s="12" t="str"/>
       <c r="C99" s="13" t="str"/>
       <c r="D99" s="12" t="str"/>
-      <c r="E99" s="12" t="str"/>
-      <c r="F99" s="14" t="str"/>
+      <c r="E99" s="14" t="str"/>
+      <c r="F99" s="12" t="str"/>
       <c r="G99" s="15" t="str"/>
     </row>
     <row r="100">
@@ -1331,8 +1331,8 @@
       <c r="B100" s="12" t="str"/>
       <c r="C100" s="13" t="str"/>
       <c r="D100" s="12" t="str"/>
-      <c r="E100" s="12" t="str"/>
-      <c r="F100" s="14" t="str"/>
+      <c r="E100" s="14" t="str"/>
+      <c r="F100" s="12" t="str"/>
       <c r="G100" s="15" t="str"/>
     </row>
     <row r="101">
@@ -1340,8 +1340,8 @@
       <c r="B101" s="12" t="str"/>
       <c r="C101" s="13" t="str"/>
       <c r="D101" s="12" t="str"/>
-      <c r="E101" s="12" t="str"/>
-      <c r="F101" s="14" t="str"/>
+      <c r="E101" s="14" t="str"/>
+      <c r="F101" s="12" t="str"/>
       <c r="G101" s="15" t="str"/>
     </row>
     <row r="102">
@@ -1349,8 +1349,8 @@
       <c r="B102" s="12" t="str"/>
       <c r="C102" s="13" t="str"/>
       <c r="D102" s="12" t="str"/>
-      <c r="E102" s="12" t="str"/>
-      <c r="F102" s="14" t="str"/>
+      <c r="E102" s="14" t="str"/>
+      <c r="F102" s="12" t="str"/>
       <c r="G102" s="15" t="str"/>
     </row>
     <row r="103">
@@ -1358,8 +1358,8 @@
       <c r="B103" s="12" t="str"/>
       <c r="C103" s="13" t="str"/>
       <c r="D103" s="12" t="str"/>
-      <c r="E103" s="12" t="str"/>
-      <c r="F103" s="14" t="str"/>
+      <c r="E103" s="14" t="str"/>
+      <c r="F103" s="12" t="str"/>
       <c r="G103" s="15" t="str"/>
     </row>
     <row r="104">
@@ -1367,8 +1367,8 @@
       <c r="B104" s="12" t="str"/>
       <c r="C104" s="13" t="str"/>
       <c r="D104" s="12" t="str"/>
-      <c r="E104" s="12" t="str"/>
-      <c r="F104" s="14" t="str"/>
+      <c r="E104" s="14" t="str"/>
+      <c r="F104" s="12" t="str"/>
       <c r="G104" s="15" t="str"/>
     </row>
     <row r="105">
@@ -1376,8 +1376,8 @@
       <c r="B105" s="12" t="str"/>
       <c r="C105" s="13" t="str"/>
       <c r="D105" s="12" t="str"/>
-      <c r="E105" s="12" t="str"/>
-      <c r="F105" s="14" t="str"/>
+      <c r="E105" s="14" t="str"/>
+      <c r="F105" s="12" t="str"/>
       <c r="G105" s="15" t="str"/>
     </row>
     <row r="106">
@@ -1385,8 +1385,8 @@
       <c r="B106" s="12" t="str"/>
       <c r="C106" s="13" t="str"/>
       <c r="D106" s="12" t="str"/>
-      <c r="E106" s="12" t="str"/>
-      <c r="F106" s="14" t="str"/>
+      <c r="E106" s="14" t="str"/>
+      <c r="F106" s="12" t="str"/>
       <c r="G106" s="15" t="str"/>
     </row>
     <row r="107">
@@ -1394,8 +1394,8 @@
       <c r="B107" s="12" t="str"/>
       <c r="C107" s="13" t="str"/>
       <c r="D107" s="12" t="str"/>
-      <c r="E107" s="12" t="str"/>
-      <c r="F107" s="14" t="str"/>
+      <c r="E107" s="14" t="str"/>
+      <c r="F107" s="12" t="str"/>
       <c r="G107" s="15" t="str"/>
     </row>
     <row r="108">
@@ -1403,8 +1403,8 @@
       <c r="B108" s="12" t="str"/>
       <c r="C108" s="13" t="str"/>
       <c r="D108" s="12" t="str"/>
-      <c r="E108" s="12" t="str"/>
-      <c r="F108" s="14" t="str"/>
+      <c r="E108" s="14" t="str"/>
+      <c r="F108" s="12" t="str"/>
       <c r="G108" s="15" t="str"/>
     </row>
     <row r="109">
@@ -1412,8 +1412,8 @@
       <c r="B109" s="12" t="str"/>
       <c r="C109" s="13" t="str"/>
       <c r="D109" s="12" t="str"/>
-      <c r="E109" s="12" t="str"/>
-      <c r="F109" s="14" t="str"/>
+      <c r="E109" s="14" t="str"/>
+      <c r="F109" s="12" t="str"/>
       <c r="G109" s="15" t="str"/>
     </row>
     <row r="110">
@@ -1421,8 +1421,8 @@
       <c r="B110" s="12" t="str"/>
       <c r="C110" s="13" t="str"/>
       <c r="D110" s="12" t="str"/>
-      <c r="E110" s="12" t="str"/>
-      <c r="F110" s="14" t="str"/>
+      <c r="E110" s="14" t="str"/>
+      <c r="F110" s="12" t="str"/>
       <c r="G110" s="15" t="str"/>
     </row>
     <row r="111">
@@ -1430,8 +1430,8 @@
       <c r="B111" s="12" t="str"/>
       <c r="C111" s="13" t="str"/>
       <c r="D111" s="12" t="str"/>
-      <c r="E111" s="12" t="str"/>
-      <c r="F111" s="14" t="str"/>
+      <c r="E111" s="14" t="str"/>
+      <c r="F111" s="12" t="str"/>
       <c r="G111" s="15" t="str"/>
     </row>
     <row r="112">
@@ -1439,8 +1439,8 @@
       <c r="B112" s="12" t="str"/>
       <c r="C112" s="13" t="str"/>
       <c r="D112" s="12" t="str"/>
-      <c r="E112" s="12" t="str"/>
-      <c r="F112" s="14" t="str"/>
+      <c r="E112" s="14" t="str"/>
+      <c r="F112" s="12" t="str"/>
       <c r="G112" s="15" t="str"/>
     </row>
     <row r="113">
@@ -1448,8 +1448,8 @@
       <c r="B113" s="12" t="str"/>
       <c r="C113" s="13" t="str"/>
       <c r="D113" s="12" t="str"/>
-      <c r="E113" s="12" t="str"/>
-      <c r="F113" s="14" t="str"/>
+      <c r="E113" s="14" t="str"/>
+      <c r="F113" s="12" t="str"/>
       <c r="G113" s="15" t="str"/>
     </row>
     <row r="114">
@@ -1457,8 +1457,8 @@
       <c r="B114" s="12" t="str"/>
       <c r="C114" s="13" t="str"/>
       <c r="D114" s="12" t="str"/>
-      <c r="E114" s="12" t="str"/>
-      <c r="F114" s="14" t="str"/>
+      <c r="E114" s="14" t="str"/>
+      <c r="F114" s="12" t="str"/>
       <c r="G114" s="15" t="str"/>
     </row>
     <row r="115">
@@ -1466,8 +1466,8 @@
       <c r="B115" s="12" t="str"/>
       <c r="C115" s="13" t="str"/>
       <c r="D115" s="12" t="str"/>
-      <c r="E115" s="12" t="str"/>
-      <c r="F115" s="14" t="str"/>
+      <c r="E115" s="14" t="str"/>
+      <c r="F115" s="12" t="str"/>
       <c r="G115" s="15" t="str"/>
     </row>
     <row r="116">
@@ -1475,8 +1475,8 @@
       <c r="B116" s="12" t="str"/>
       <c r="C116" s="13" t="str"/>
       <c r="D116" s="12" t="str"/>
-      <c r="E116" s="12" t="str"/>
-      <c r="F116" s="14" t="str"/>
+      <c r="E116" s="14" t="str"/>
+      <c r="F116" s="12" t="str"/>
       <c r="G116" s="15" t="str"/>
     </row>
     <row r="117">
@@ -1484,8 +1484,8 @@
       <c r="B117" s="12" t="str"/>
       <c r="C117" s="13" t="str"/>
       <c r="D117" s="12" t="str"/>
-      <c r="E117" s="12" t="str"/>
-      <c r="F117" s="14" t="str"/>
+      <c r="E117" s="14" t="str"/>
+      <c r="F117" s="12" t="str"/>
       <c r="G117" s="15" t="str"/>
     </row>
     <row r="118">
@@ -1493,8 +1493,8 @@
       <c r="B118" s="12" t="str"/>
       <c r="C118" s="13" t="str"/>
       <c r="D118" s="12" t="str"/>
-      <c r="E118" s="12" t="str"/>
-      <c r="F118" s="14" t="str"/>
+      <c r="E118" s="14" t="str"/>
+      <c r="F118" s="12" t="str"/>
       <c r="G118" s="15" t="str"/>
     </row>
     <row r="119">
@@ -1502,8 +1502,8 @@
       <c r="B119" s="12" t="str"/>
       <c r="C119" s="13" t="str"/>
       <c r="D119" s="12" t="str"/>
-      <c r="E119" s="12" t="str"/>
-      <c r="F119" s="14" t="str"/>
+      <c r="E119" s="14" t="str"/>
+      <c r="F119" s="12" t="str"/>
       <c r="G119" s="15" t="str"/>
     </row>
     <row r="120">
@@ -1511,8 +1511,8 @@
       <c r="B120" s="12" t="str"/>
       <c r="C120" s="13" t="str"/>
       <c r="D120" s="12" t="str"/>
-      <c r="E120" s="12" t="str"/>
-      <c r="F120" s="14" t="str"/>
+      <c r="E120" s="14" t="str"/>
+      <c r="F120" s="12" t="str"/>
       <c r="G120" s="15" t="str"/>
     </row>
     <row r="121">
@@ -1520,8 +1520,8 @@
       <c r="B121" s="12" t="str"/>
       <c r="C121" s="13" t="str"/>
       <c r="D121" s="12" t="str"/>
-      <c r="E121" s="12" t="str"/>
-      <c r="F121" s="14" t="str"/>
+      <c r="E121" s="14" t="str"/>
+      <c r="F121" s="12" t="str"/>
       <c r="G121" s="15" t="str"/>
     </row>
     <row r="122">
@@ -1529,8 +1529,8 @@
       <c r="B122" s="12" t="str"/>
       <c r="C122" s="13" t="str"/>
       <c r="D122" s="12" t="str"/>
-      <c r="E122" s="12" t="str"/>
-      <c r="F122" s="14" t="str"/>
+      <c r="E122" s="14" t="str"/>
+      <c r="F122" s="12" t="str"/>
       <c r="G122" s="15" t="str"/>
     </row>
     <row r="123">
@@ -1538,8 +1538,8 @@
       <c r="B123" s="12" t="str"/>
       <c r="C123" s="13" t="str"/>
       <c r="D123" s="12" t="str"/>
-      <c r="E123" s="12" t="str"/>
-      <c r="F123" s="14" t="str"/>
+      <c r="E123" s="14" t="str"/>
+      <c r="F123" s="12" t="str"/>
       <c r="G123" s="15" t="str"/>
     </row>
     <row r="124">
@@ -1547,8 +1547,8 @@
       <c r="B124" s="12" t="str"/>
       <c r="C124" s="13" t="str"/>
       <c r="D124" s="12" t="str"/>
-      <c r="E124" s="12" t="str"/>
-      <c r="F124" s="14" t="str"/>
+      <c r="E124" s="14" t="str"/>
+      <c r="F124" s="12" t="str"/>
       <c r="G124" s="15" t="str"/>
     </row>
     <row r="125">
@@ -1556,8 +1556,8 @@
       <c r="B125" s="12" t="str"/>
       <c r="C125" s="13" t="str"/>
       <c r="D125" s="12" t="str"/>
-      <c r="E125" s="12" t="str"/>
-      <c r="F125" s="14" t="str"/>
+      <c r="E125" s="14" t="str"/>
+      <c r="F125" s="12" t="str"/>
       <c r="G125" s="15" t="str"/>
     </row>
     <row r="126">
@@ -1565,8 +1565,8 @@
       <c r="B126" s="12" t="str"/>
       <c r="C126" s="13" t="str"/>
       <c r="D126" s="12" t="str"/>
-      <c r="E126" s="12" t="str"/>
-      <c r="F126" s="14" t="str"/>
+      <c r="E126" s="14" t="str"/>
+      <c r="F126" s="12" t="str"/>
       <c r="G126" s="15" t="str"/>
     </row>
     <row r="127">
@@ -1574,8 +1574,8 @@
       <c r="B127" s="12" t="str"/>
       <c r="C127" s="13" t="str"/>
       <c r="D127" s="12" t="str"/>
-      <c r="E127" s="12" t="str"/>
-      <c r="F127" s="14" t="str"/>
+      <c r="E127" s="14" t="str"/>
+      <c r="F127" s="12" t="str"/>
       <c r="G127" s="15" t="str"/>
     </row>
     <row r="128">
@@ -1583,8 +1583,8 @@
       <c r="B128" s="12" t="str"/>
       <c r="C128" s="13" t="str"/>
       <c r="D128" s="12" t="str"/>
-      <c r="E128" s="12" t="str"/>
-      <c r="F128" s="14" t="str"/>
+      <c r="E128" s="14" t="str"/>
+      <c r="F128" s="12" t="str"/>
       <c r="G128" s="15" t="str"/>
     </row>
     <row r="129">
@@ -1592,8 +1592,8 @@
       <c r="B129" s="12" t="str"/>
       <c r="C129" s="13" t="str"/>
       <c r="D129" s="12" t="str"/>
-      <c r="E129" s="12" t="str"/>
-      <c r="F129" s="14" t="str"/>
+      <c r="E129" s="14" t="str"/>
+      <c r="F129" s="12" t="str"/>
       <c r="G129" s="15" t="str"/>
     </row>
     <row r="130">
@@ -1601,8 +1601,8 @@
       <c r="B130" s="12" t="str"/>
       <c r="C130" s="13" t="str"/>
       <c r="D130" s="12" t="str"/>
-      <c r="E130" s="12" t="str"/>
-      <c r="F130" s="14" t="str"/>
+      <c r="E130" s="14" t="str"/>
+      <c r="F130" s="12" t="str"/>
       <c r="G130" s="15" t="str"/>
     </row>
     <row r="131">
@@ -1610,8 +1610,8 @@
       <c r="B131" s="12" t="str"/>
       <c r="C131" s="13" t="str"/>
       <c r="D131" s="12" t="str"/>
-      <c r="E131" s="12" t="str"/>
-      <c r="F131" s="14" t="str"/>
+      <c r="E131" s="14" t="str"/>
+      <c r="F131" s="12" t="str"/>
       <c r="G131" s="15" t="str"/>
     </row>
     <row r="132">
@@ -1619,8 +1619,8 @@
       <c r="B132" s="12" t="str"/>
       <c r="C132" s="13" t="str"/>
       <c r="D132" s="12" t="str"/>
-      <c r="E132" s="12" t="str"/>
-      <c r="F132" s="14" t="str"/>
+      <c r="E132" s="14" t="str"/>
+      <c r="F132" s="12" t="str"/>
       <c r="G132" s="15" t="str"/>
     </row>
     <row r="133">
@@ -1628,8 +1628,8 @@
       <c r="B133" s="12" t="str"/>
       <c r="C133" s="13" t="str"/>
       <c r="D133" s="12" t="str"/>
-      <c r="E133" s="12" t="str"/>
-      <c r="F133" s="14" t="str"/>
+      <c r="E133" s="14" t="str"/>
+      <c r="F133" s="12" t="str"/>
       <c r="G133" s="15" t="str"/>
     </row>
     <row r="134">
@@ -1637,8 +1637,8 @@
       <c r="B134" s="12" t="str"/>
       <c r="C134" s="13" t="str"/>
       <c r="D134" s="12" t="str"/>
-      <c r="E134" s="12" t="str"/>
-      <c r="F134" s="14" t="str"/>
+      <c r="E134" s="14" t="str"/>
+      <c r="F134" s="12" t="str"/>
       <c r="G134" s="15" t="str"/>
     </row>
     <row r="135">
@@ -1646,8 +1646,8 @@
       <c r="B135" s="12" t="str"/>
       <c r="C135" s="13" t="str"/>
       <c r="D135" s="12" t="str"/>
-      <c r="E135" s="12" t="str"/>
-      <c r="F135" s="14" t="str"/>
+      <c r="E135" s="14" t="str"/>
+      <c r="F135" s="12" t="str"/>
       <c r="G135" s="15" t="str"/>
     </row>
     <row r="136">
@@ -1655,8 +1655,8 @@
       <c r="B136" s="12" t="str"/>
       <c r="C136" s="13" t="str"/>
       <c r="D136" s="12" t="str"/>
-      <c r="E136" s="12" t="str"/>
-      <c r="F136" s="14" t="str"/>
+      <c r="E136" s="14" t="str"/>
+      <c r="F136" s="12" t="str"/>
       <c r="G136" s="15" t="str"/>
     </row>
     <row r="137">
@@ -1664,8 +1664,8 @@
       <c r="B137" s="12" t="str"/>
       <c r="C137" s="13" t="str"/>
       <c r="D137" s="12" t="str"/>
-      <c r="E137" s="12" t="str"/>
-      <c r="F137" s="14" t="str"/>
+      <c r="E137" s="14" t="str"/>
+      <c r="F137" s="12" t="str"/>
       <c r="G137" s="15" t="str"/>
     </row>
     <row r="138">
@@ -1673,8 +1673,8 @@
       <c r="B138" s="12" t="str"/>
       <c r="C138" s="13" t="str"/>
       <c r="D138" s="12" t="str"/>
-      <c r="E138" s="12" t="str"/>
-      <c r="F138" s="14" t="str"/>
+      <c r="E138" s="14" t="str"/>
+      <c r="F138" s="12" t="str"/>
       <c r="G138" s="15" t="str"/>
     </row>
     <row r="139">
@@ -1682,8 +1682,8 @@
       <c r="B139" s="12" t="str"/>
       <c r="C139" s="13" t="str"/>
       <c r="D139" s="12" t="str"/>
-      <c r="E139" s="12" t="str"/>
-      <c r="F139" s="14" t="str"/>
+      <c r="E139" s="14" t="str"/>
+      <c r="F139" s="12" t="str"/>
       <c r="G139" s="15" t="str"/>
     </row>
     <row r="140">
@@ -1691,8 +1691,8 @@
       <c r="B140" s="12" t="str"/>
       <c r="C140" s="13" t="str"/>
       <c r="D140" s="12" t="str"/>
-      <c r="E140" s="12" t="str"/>
-      <c r="F140" s="14" t="str"/>
+      <c r="E140" s="14" t="str"/>
+      <c r="F140" s="12" t="str"/>
       <c r="G140" s="15" t="str"/>
     </row>
     <row r="141">
@@ -1700,8 +1700,8 @@
       <c r="B141" s="12" t="str"/>
       <c r="C141" s="13" t="str"/>
       <c r="D141" s="12" t="str"/>
-      <c r="E141" s="12" t="str"/>
-      <c r="F141" s="14" t="str"/>
+      <c r="E141" s="14" t="str"/>
+      <c r="F141" s="12" t="str"/>
       <c r="G141" s="15" t="str"/>
     </row>
     <row r="142">
@@ -1709,8 +1709,8 @@
       <c r="B142" s="12" t="str"/>
       <c r="C142" s="13" t="str"/>
       <c r="D142" s="12" t="str"/>
-      <c r="E142" s="12" t="str"/>
-      <c r="F142" s="14" t="str"/>
+      <c r="E142" s="14" t="str"/>
+      <c r="F142" s="12" t="str"/>
       <c r="G142" s="15" t="str"/>
     </row>
     <row r="143">
@@ -1718,8 +1718,8 @@
       <c r="B143" s="12" t="str"/>
       <c r="C143" s="13" t="str"/>
       <c r="D143" s="12" t="str"/>
-      <c r="E143" s="12" t="str"/>
-      <c r="F143" s="14" t="str"/>
+      <c r="E143" s="14" t="str"/>
+      <c r="F143" s="12" t="str"/>
       <c r="G143" s="15" t="str"/>
     </row>
     <row r="144">
@@ -1727,8 +1727,8 @@
       <c r="B144" s="12" t="str"/>
       <c r="C144" s="13" t="str"/>
       <c r="D144" s="12" t="str"/>
-      <c r="E144" s="12" t="str"/>
-      <c r="F144" s="14" t="str"/>
+      <c r="E144" s="14" t="str"/>
+      <c r="F144" s="12" t="str"/>
       <c r="G144" s="15" t="str"/>
     </row>
     <row r="145">
@@ -1736,8 +1736,8 @@
       <c r="B145" s="12" t="str"/>
       <c r="C145" s="13" t="str"/>
       <c r="D145" s="12" t="str"/>
-      <c r="E145" s="12" t="str"/>
-      <c r="F145" s="14" t="str"/>
+      <c r="E145" s="14" t="str"/>
+      <c r="F145" s="12" t="str"/>
       <c r="G145" s="15" t="str"/>
     </row>
     <row r="146">
@@ -1745,8 +1745,8 @@
       <c r="B146" s="12" t="str"/>
       <c r="C146" s="13" t="str"/>
       <c r="D146" s="12" t="str"/>
-      <c r="E146" s="12" t="str"/>
-      <c r="F146" s="14" t="str"/>
+      <c r="E146" s="14" t="str"/>
+      <c r="F146" s="12" t="str"/>
       <c r="G146" s="15" t="str"/>
     </row>
     <row r="147">
@@ -1754,8 +1754,8 @@
       <c r="B147" s="12" t="str"/>
       <c r="C147" s="13" t="str"/>
       <c r="D147" s="12" t="str"/>
-      <c r="E147" s="12" t="str"/>
-      <c r="F147" s="14" t="str"/>
+      <c r="E147" s="14" t="str"/>
+      <c r="F147" s="12" t="str"/>
       <c r="G147" s="15" t="str"/>
     </row>
     <row r="148">
@@ -1763,8 +1763,8 @@
       <c r="B148" s="12" t="str"/>
       <c r="C148" s="13" t="str"/>
       <c r="D148" s="12" t="str"/>
-      <c r="E148" s="12" t="str"/>
-      <c r="F148" s="14" t="str"/>
+      <c r="E148" s="14" t="str"/>
+      <c r="F148" s="12" t="str"/>
       <c r="G148" s="15" t="str"/>
     </row>
     <row r="149">
@@ -1772,8 +1772,8 @@
       <c r="B149" s="12" t="str"/>
       <c r="C149" s="13" t="str"/>
       <c r="D149" s="12" t="str"/>
-      <c r="E149" s="12" t="str"/>
-      <c r="F149" s="14" t="str"/>
+      <c r="E149" s="14" t="str"/>
+      <c r="F149" s="12" t="str"/>
       <c r="G149" s="15" t="str"/>
     </row>
     <row r="150">
@@ -1781,8 +1781,8 @@
       <c r="B150" s="12" t="str"/>
       <c r="C150" s="13" t="str"/>
       <c r="D150" s="12" t="str"/>
-      <c r="E150" s="12" t="str"/>
-      <c r="F150" s="14" t="str"/>
+      <c r="E150" s="14" t="str"/>
+      <c r="F150" s="12" t="str"/>
       <c r="G150" s="15" t="str"/>
     </row>
     <row r="151">
@@ -1790,8 +1790,8 @@
       <c r="B151" s="12" t="str"/>
       <c r="C151" s="13" t="str"/>
       <c r="D151" s="12" t="str"/>
-      <c r="E151" s="12" t="str"/>
-      <c r="F151" s="14" t="str"/>
+      <c r="E151" s="14" t="str"/>
+      <c r="F151" s="12" t="str"/>
       <c r="G151" s="15" t="str"/>
     </row>
     <row r="152">
@@ -1799,8 +1799,8 @@
       <c r="B152" s="12" t="str"/>
       <c r="C152" s="13" t="str"/>
       <c r="D152" s="12" t="str"/>
-      <c r="E152" s="12" t="str"/>
-      <c r="F152" s="14" t="str"/>
+      <c r="E152" s="14" t="str"/>
+      <c r="F152" s="12" t="str"/>
       <c r="G152" s="15" t="str"/>
     </row>
     <row r="153">
@@ -1808,8 +1808,8 @@
       <c r="B153" s="12" t="str"/>
       <c r="C153" s="13" t="str"/>
       <c r="D153" s="12" t="str"/>
-      <c r="E153" s="12" t="str"/>
-      <c r="F153" s="14" t="str"/>
+      <c r="E153" s="14" t="str"/>
+      <c r="F153" s="12" t="str"/>
       <c r="G153" s="15" t="str"/>
     </row>
     <row r="154">
@@ -1817,8 +1817,8 @@
       <c r="B154" s="12" t="str"/>
       <c r="C154" s="13" t="str"/>
       <c r="D154" s="12" t="str"/>
-      <c r="E154" s="12" t="str"/>
-      <c r="F154" s="14" t="str"/>
+      <c r="E154" s="14" t="str"/>
+      <c r="F154" s="12" t="str"/>
       <c r="G154" s="15" t="str"/>
     </row>
     <row r="155">
@@ -1826,8 +1826,8 @@
       <c r="B155" s="12" t="str"/>
       <c r="C155" s="13" t="str"/>
       <c r="D155" s="12" t="str"/>
-      <c r="E155" s="12" t="str"/>
-      <c r="F155" s="14" t="str"/>
+      <c r="E155" s="14" t="str"/>
+      <c r="F155" s="12" t="str"/>
       <c r="G155" s="15" t="str"/>
     </row>
     <row r="156">
@@ -1835,8 +1835,8 @@
       <c r="B156" s="12" t="str"/>
       <c r="C156" s="13" t="str"/>
       <c r="D156" s="12" t="str"/>
-      <c r="E156" s="12" t="str"/>
-      <c r="F156" s="14" t="str"/>
+      <c r="E156" s="14" t="str"/>
+      <c r="F156" s="12" t="str"/>
       <c r="G156" s="15" t="str"/>
     </row>
     <row r="157">
@@ -1844,8 +1844,8 @@
       <c r="B157" s="12" t="str"/>
       <c r="C157" s="13" t="str"/>
       <c r="D157" s="12" t="str"/>
-      <c r="E157" s="12" t="str"/>
-      <c r="F157" s="14" t="str"/>
+      <c r="E157" s="14" t="str"/>
+      <c r="F157" s="12" t="str"/>
       <c r="G157" s="15" t="str"/>
     </row>
     <row r="158">
@@ -1853,8 +1853,8 @@
       <c r="B158" s="12" t="str"/>
       <c r="C158" s="13" t="str"/>
       <c r="D158" s="12" t="str"/>
-      <c r="E158" s="12" t="str"/>
-      <c r="F158" s="14" t="str"/>
+      <c r="E158" s="14" t="str"/>
+      <c r="F158" s="12" t="str"/>
       <c r="G158" s="15" t="str"/>
     </row>
     <row r="159">
@@ -1862,8 +1862,8 @@
       <c r="B159" s="12" t="str"/>
       <c r="C159" s="13" t="str"/>
       <c r="D159" s="12" t="str"/>
-      <c r="E159" s="12" t="str"/>
-      <c r="F159" s="14" t="str"/>
+      <c r="E159" s="14" t="str"/>
+      <c r="F159" s="12" t="str"/>
       <c r="G159" s="15" t="str"/>
     </row>
     <row r="160">
@@ -1871,8 +1871,8 @@
       <c r="B160" s="12" t="str"/>
       <c r="C160" s="13" t="str"/>
       <c r="D160" s="12" t="str"/>
-      <c r="E160" s="12" t="str"/>
-      <c r="F160" s="14" t="str"/>
+      <c r="E160" s="14" t="str"/>
+      <c r="F160" s="12" t="str"/>
       <c r="G160" s="15" t="str"/>
     </row>
     <row r="161">
@@ -1880,8 +1880,8 @@
       <c r="B161" s="12" t="str"/>
       <c r="C161" s="13" t="str"/>
       <c r="D161" s="12" t="str"/>
-      <c r="E161" s="12" t="str"/>
-      <c r="F161" s="14" t="str"/>
+      <c r="E161" s="14" t="str"/>
+      <c r="F161" s="12" t="str"/>
       <c r="G161" s="15" t="str"/>
     </row>
     <row r="162">
@@ -1889,8 +1889,8 @@
       <c r="B162" s="12" t="str"/>
       <c r="C162" s="13" t="str"/>
       <c r="D162" s="12" t="str"/>
-      <c r="E162" s="12" t="str"/>
-      <c r="F162" s="14" t="str"/>
+      <c r="E162" s="14" t="str"/>
+      <c r="F162" s="12" t="str"/>
       <c r="G162" s="15" t="str"/>
     </row>
     <row r="163">
@@ -1898,8 +1898,8 @@
       <c r="B163" s="12" t="str"/>
       <c r="C163" s="13" t="str"/>
       <c r="D163" s="12" t="str"/>
-      <c r="E163" s="12" t="str"/>
-      <c r="F163" s="14" t="str"/>
+      <c r="E163" s="14" t="str"/>
+      <c r="F163" s="12" t="str"/>
       <c r="G163" s="15" t="str"/>
     </row>
     <row r="164">
@@ -1907,8 +1907,8 @@
       <c r="B164" s="12" t="str"/>
       <c r="C164" s="13" t="str"/>
       <c r="D164" s="12" t="str"/>
-      <c r="E164" s="12" t="str"/>
-      <c r="F164" s="14" t="str"/>
+      <c r="E164" s="14" t="str"/>
+      <c r="F164" s="12" t="str"/>
       <c r="G164" s="15" t="str"/>
     </row>
     <row r="165">
@@ -1916,8 +1916,8 @@
       <c r="B165" s="12" t="str"/>
       <c r="C165" s="13" t="str"/>
       <c r="D165" s="12" t="str"/>
-      <c r="E165" s="12" t="str"/>
-      <c r="F165" s="14" t="str"/>
+      <c r="E165" s="14" t="str"/>
+      <c r="F165" s="12" t="str"/>
       <c r="G165" s="15" t="str"/>
     </row>
     <row r="166">
@@ -1925,8 +1925,8 @@
       <c r="B166" s="12" t="str"/>
       <c r="C166" s="13" t="str"/>
       <c r="D166" s="12" t="str"/>
-      <c r="E166" s="12" t="str"/>
-      <c r="F166" s="14" t="str"/>
+      <c r="E166" s="14" t="str"/>
+      <c r="F166" s="12" t="str"/>
       <c r="G166" s="15" t="str"/>
     </row>
     <row r="167">
@@ -1934,8 +1934,8 @@
       <c r="B167" s="12" t="str"/>
       <c r="C167" s="13" t="str"/>
       <c r="D167" s="12" t="str"/>
-      <c r="E167" s="12" t="str"/>
-      <c r="F167" s="14" t="str"/>
+      <c r="E167" s="14" t="str"/>
+      <c r="F167" s="12" t="str"/>
       <c r="G167" s="15" t="str"/>
     </row>
     <row r="168">
@@ -1943,8 +1943,8 @@
       <c r="B168" s="12" t="str"/>
       <c r="C168" s="13" t="str"/>
       <c r="D168" s="12" t="str"/>
-      <c r="E168" s="12" t="str"/>
-      <c r="F168" s="14" t="str"/>
+      <c r="E168" s="14" t="str"/>
+      <c r="F168" s="12" t="str"/>
       <c r="G168" s="15" t="str"/>
     </row>
     <row r="169">
@@ -1952,8 +1952,8 @@
       <c r="B169" s="12" t="str"/>
       <c r="C169" s="13" t="str"/>
       <c r="D169" s="12" t="str"/>
-      <c r="E169" s="12" t="str"/>
-      <c r="F169" s="14" t="str"/>
+      <c r="E169" s="14" t="str"/>
+      <c r="F169" s="12" t="str"/>
       <c r="G169" s="15" t="str"/>
     </row>
     <row r="170">
@@ -1961,8 +1961,8 @@
       <c r="B170" s="12" t="str"/>
       <c r="C170" s="13" t="str"/>
       <c r="D170" s="12" t="str"/>
-      <c r="E170" s="12" t="str"/>
-      <c r="F170" s="14" t="str"/>
+      <c r="E170" s="14" t="str"/>
+      <c r="F170" s="12" t="str"/>
       <c r="G170" s="15" t="str"/>
     </row>
     <row r="171">
@@ -1970,8 +1970,8 @@
       <c r="B171" s="12" t="str"/>
       <c r="C171" s="13" t="str"/>
       <c r="D171" s="12" t="str"/>
-      <c r="E171" s="12" t="str"/>
-      <c r="F171" s="14" t="str"/>
+      <c r="E171" s="14" t="str"/>
+      <c r="F171" s="12" t="str"/>
       <c r="G171" s="15" t="str"/>
     </row>
     <row r="172">
@@ -1979,8 +1979,8 @@
       <c r="B172" s="12" t="str"/>
       <c r="C172" s="13" t="str"/>
       <c r="D172" s="12" t="str"/>
-      <c r="E172" s="12" t="str"/>
-      <c r="F172" s="14" t="str"/>
+      <c r="E172" s="14" t="str"/>
+      <c r="F172" s="12" t="str"/>
       <c r="G172" s="15" t="str"/>
     </row>
     <row r="173">
@@ -1988,8 +1988,8 @@
       <c r="B173" s="12" t="str"/>
       <c r="C173" s="13" t="str"/>
       <c r="D173" s="12" t="str"/>
-      <c r="E173" s="12" t="str"/>
-      <c r="F173" s="14" t="str"/>
+      <c r="E173" s="14" t="str"/>
+      <c r="F173" s="12" t="str"/>
       <c r="G173" s="15" t="str"/>
     </row>
     <row r="174">
@@ -1997,8 +1997,8 @@
       <c r="B174" s="12" t="str"/>
       <c r="C174" s="13" t="str"/>
       <c r="D174" s="12" t="str"/>
-      <c r="E174" s="12" t="str"/>
-      <c r="F174" s="14" t="str"/>
+      <c r="E174" s="14" t="str"/>
+      <c r="F174" s="12" t="str"/>
       <c r="G174" s="15" t="str"/>
     </row>
     <row r="175">
@@ -2006,8 +2006,8 @@
       <c r="B175" s="12" t="str"/>
       <c r="C175" s="13" t="str"/>
       <c r="D175" s="12" t="str"/>
-      <c r="E175" s="12" t="str"/>
-      <c r="F175" s="14" t="str"/>
+      <c r="E175" s="14" t="str"/>
+      <c r="F175" s="12" t="str"/>
       <c r="G175" s="15" t="str"/>
     </row>
     <row r="176">
@@ -2015,8 +2015,8 @@
       <c r="B176" s="12" t="str"/>
       <c r="C176" s="13" t="str"/>
       <c r="D176" s="12" t="str"/>
-      <c r="E176" s="12" t="str"/>
-      <c r="F176" s="14" t="str"/>
+      <c r="E176" s="14" t="str"/>
+      <c r="F176" s="12" t="str"/>
       <c r="G176" s="15" t="str"/>
     </row>
     <row r="177">
@@ -2024,8 +2024,8 @@
       <c r="B177" s="12" t="str"/>
       <c r="C177" s="13" t="str"/>
       <c r="D177" s="12" t="str"/>
-      <c r="E177" s="12" t="str"/>
-      <c r="F177" s="14" t="str"/>
+      <c r="E177" s="14" t="str"/>
+      <c r="F177" s="12" t="str"/>
       <c r="G177" s="15" t="str"/>
     </row>
     <row r="178">
@@ -2033,8 +2033,8 @@
       <c r="B178" s="12" t="str"/>
       <c r="C178" s="13" t="str"/>
       <c r="D178" s="12" t="str"/>
-      <c r="E178" s="12" t="str"/>
-      <c r="F178" s="14" t="str"/>
+      <c r="E178" s="14" t="str"/>
+      <c r="F178" s="12" t="str"/>
       <c r="G178" s="15" t="str"/>
     </row>
     <row r="179">
@@ -2042,8 +2042,8 @@
       <c r="B179" s="12" t="str"/>
       <c r="C179" s="13" t="str"/>
       <c r="D179" s="12" t="str"/>
-      <c r="E179" s="12" t="str"/>
-      <c r="F179" s="14" t="str"/>
+      <c r="E179" s="14" t="str"/>
+      <c r="F179" s="12" t="str"/>
       <c r="G179" s="15" t="str"/>
     </row>
     <row r="180">
@@ -2051,8 +2051,8 @@
       <c r="B180" s="12" t="str"/>
       <c r="C180" s="13" t="str"/>
       <c r="D180" s="12" t="str"/>
-      <c r="E180" s="12" t="str"/>
-      <c r="F180" s="14" t="str"/>
+      <c r="E180" s="14" t="str"/>
+      <c r="F180" s="12" t="str"/>
       <c r="G180" s="15" t="str"/>
     </row>
     <row r="181">
@@ -2060,8 +2060,8 @@
       <c r="B181" s="12" t="str"/>
       <c r="C181" s="13" t="str"/>
       <c r="D181" s="12" t="str"/>
-      <c r="E181" s="12" t="str"/>
-      <c r="F181" s="14" t="str"/>
+      <c r="E181" s="14" t="str"/>
+      <c r="F181" s="12" t="str"/>
       <c r="G181" s="15" t="str"/>
     </row>
     <row r="182">
@@ -2069,8 +2069,8 @@
       <c r="B182" s="12" t="str"/>
       <c r="C182" s="13" t="str"/>
       <c r="D182" s="12" t="str"/>
-      <c r="E182" s="12" t="str"/>
-      <c r="F182" s="14" t="str"/>
+      <c r="E182" s="14" t="str"/>
+      <c r="F182" s="12" t="str"/>
       <c r="G182" s="15" t="str"/>
     </row>
     <row r="183">
@@ -2078,8 +2078,8 @@
       <c r="B183" s="12" t="str"/>
       <c r="C183" s="13" t="str"/>
       <c r="D183" s="12" t="str"/>
-      <c r="E183" s="12" t="str"/>
-      <c r="F183" s="14" t="str"/>
+      <c r="E183" s="14" t="str"/>
+      <c r="F183" s="12" t="str"/>
       <c r="G183" s="15" t="str"/>
     </row>
     <row r="184">
@@ -2087,8 +2087,8 @@
       <c r="B184" s="12" t="str"/>
       <c r="C184" s="13" t="str"/>
       <c r="D184" s="12" t="str"/>
-      <c r="E184" s="12" t="str"/>
-      <c r="F184" s="14" t="str"/>
+      <c r="E184" s="14" t="str"/>
+      <c r="F184" s="12" t="str"/>
       <c r="G184" s="15" t="str"/>
     </row>
     <row r="185">
@@ -2096,8 +2096,8 @@
       <c r="B185" s="12" t="str"/>
       <c r="C185" s="13" t="str"/>
       <c r="D185" s="12" t="str"/>
-      <c r="E185" s="12" t="str"/>
-      <c r="F185" s="14" t="str"/>
+      <c r="E185" s="14" t="str"/>
+      <c r="F185" s="12" t="str"/>
       <c r="G185" s="15" t="str"/>
     </row>
     <row r="186">
@@ -2105,8 +2105,8 @@
       <c r="B186" s="12" t="str"/>
       <c r="C186" s="13" t="str"/>
       <c r="D186" s="12" t="str"/>
-      <c r="E186" s="12" t="str"/>
-      <c r="F186" s="14" t="str"/>
+      <c r="E186" s="14" t="str"/>
+      <c r="F186" s="12" t="str"/>
       <c r="G186" s="15" t="str"/>
     </row>
     <row r="187">
@@ -2114,8 +2114,8 @@
       <c r="B187" s="12" t="str"/>
       <c r="C187" s="13" t="str"/>
       <c r="D187" s="12" t="str"/>
-      <c r="E187" s="12" t="str"/>
-      <c r="F187" s="14" t="str"/>
+      <c r="E187" s="14" t="str"/>
+      <c r="F187" s="12" t="str"/>
       <c r="G187" s="15" t="str"/>
     </row>
     <row r="188">
@@ -2123,8 +2123,8 @@
       <c r="B188" s="12" t="str"/>
       <c r="C188" s="13" t="str"/>
       <c r="D188" s="12" t="str"/>
-      <c r="E188" s="12" t="str"/>
-      <c r="F188" s="14" t="str"/>
+      <c r="E188" s="14" t="str"/>
+      <c r="F188" s="12" t="str"/>
       <c r="G188" s="15" t="str"/>
     </row>
     <row r="189">
@@ -2132,8 +2132,8 @@
       <c r="B189" s="12" t="str"/>
       <c r="C189" s="13" t="str"/>
       <c r="D189" s="12" t="str"/>
-      <c r="E189" s="12" t="str"/>
-      <c r="F189" s="14" t="str"/>
+      <c r="E189" s="14" t="str"/>
+      <c r="F189" s="12" t="str"/>
       <c r="G189" s="15" t="str"/>
     </row>
     <row r="190">
@@ -2141,8 +2141,8 @@
       <c r="B190" s="12" t="str"/>
       <c r="C190" s="13" t="str"/>
       <c r="D190" s="12" t="str"/>
-      <c r="E190" s="12" t="str"/>
-      <c r="F190" s="14" t="str"/>
+      <c r="E190" s="14" t="str"/>
+      <c r="F190" s="12" t="str"/>
       <c r="G190" s="15" t="str"/>
     </row>
     <row r="191">
@@ -2150,8 +2150,8 @@
       <c r="B191" s="12" t="str"/>
       <c r="C191" s="13" t="str"/>
       <c r="D191" s="12" t="str"/>
-      <c r="E191" s="12" t="str"/>
-      <c r="F191" s="14" t="str"/>
+      <c r="E191" s="14" t="str"/>
+      <c r="F191" s="12" t="str"/>
       <c r="G191" s="15" t="str"/>
     </row>
     <row r="192">
@@ -2159,8 +2159,8 @@
       <c r="B192" s="12" t="str"/>
       <c r="C192" s="13" t="str"/>
       <c r="D192" s="12" t="str"/>
-      <c r="E192" s="12" t="str"/>
-      <c r="F192" s="14" t="str"/>
+      <c r="E192" s="14" t="str"/>
+      <c r="F192" s="12" t="str"/>
       <c r="G192" s="15" t="str"/>
     </row>
     <row r="193">
@@ -2168,8 +2168,8 @@
       <c r="B193" s="12" t="str"/>
       <c r="C193" s="13" t="str"/>
       <c r="D193" s="12" t="str"/>
-      <c r="E193" s="12" t="str"/>
-      <c r="F193" s="14" t="str"/>
+      <c r="E193" s="14" t="str"/>
+      <c r="F193" s="12" t="str"/>
       <c r="G193" s="15" t="str"/>
     </row>
     <row r="194">
@@ -2177,8 +2177,8 @@
       <c r="B194" s="12" t="str"/>
       <c r="C194" s="13" t="str"/>
       <c r="D194" s="12" t="str"/>
-      <c r="E194" s="12" t="str"/>
-      <c r="F194" s="14" t="str"/>
+      <c r="E194" s="14" t="str"/>
+      <c r="F194" s="12" t="str"/>
       <c r="G194" s="15" t="str"/>
     </row>
     <row r="195">
@@ -2186,8 +2186,8 @@
       <c r="B195" s="12" t="str"/>
       <c r="C195" s="13" t="str"/>
       <c r="D195" s="12" t="str"/>
-      <c r="E195" s="12" t="str"/>
-      <c r="F195" s="14" t="str"/>
+      <c r="E195" s="14" t="str"/>
+      <c r="F195" s="12" t="str"/>
       <c r="G195" s="15" t="str"/>
     </row>
     <row r="196">
@@ -2195,8 +2195,8 @@
       <c r="B196" s="12" t="str"/>
       <c r="C196" s="13" t="str"/>
       <c r="D196" s="12" t="str"/>
-      <c r="E196" s="12" t="str"/>
-      <c r="F196" s="14" t="str"/>
+      <c r="E196" s="14" t="str"/>
+      <c r="F196" s="12" t="str"/>
       <c r="G196" s="15" t="str"/>
     </row>
     <row r="197">
@@ -2204,8 +2204,8 @@
       <c r="B197" s="12" t="str"/>
       <c r="C197" s="13" t="str"/>
       <c r="D197" s="12" t="str"/>
-      <c r="E197" s="12" t="str"/>
-      <c r="F197" s="14" t="str"/>
+      <c r="E197" s="14" t="str"/>
+      <c r="F197" s="12" t="str"/>
       <c r="G197" s="15" t="str"/>
     </row>
     <row r="198">
@@ -2213,8 +2213,8 @@
       <c r="B198" s="12" t="str"/>
       <c r="C198" s="13" t="str"/>
       <c r="D198" s="12" t="str"/>
-      <c r="E198" s="12" t="str"/>
-      <c r="F198" s="14" t="str"/>
+      <c r="E198" s="14" t="str"/>
+      <c r="F198" s="12" t="str"/>
       <c r="G198" s="15" t="str"/>
     </row>
     <row r="199">
@@ -2222,8 +2222,8 @@
       <c r="B199" s="12" t="str"/>
       <c r="C199" s="13" t="str"/>
       <c r="D199" s="12" t="str"/>
-      <c r="E199" s="12" t="str"/>
-      <c r="F199" s="14" t="str"/>
+      <c r="E199" s="14" t="str"/>
+      <c r="F199" s="12" t="str"/>
       <c r="G199" s="15" t="str"/>
     </row>
     <row r="200">
@@ -2231,8 +2231,8 @@
       <c r="B200" s="12" t="str"/>
       <c r="C200" s="13" t="str"/>
       <c r="D200" s="12" t="str"/>
-      <c r="E200" s="12" t="str"/>
-      <c r="F200" s="14" t="str"/>
+      <c r="E200" s="14" t="str"/>
+      <c r="F200" s="12" t="str"/>
       <c r="G200" s="15" t="str"/>
     </row>
     <row r="201">
@@ -2240,8 +2240,8 @@
       <c r="B201" s="12" t="str"/>
       <c r="C201" s="13" t="str"/>
       <c r="D201" s="12" t="str"/>
-      <c r="E201" s="12" t="str"/>
-      <c r="F201" s="14" t="str"/>
+      <c r="E201" s="14" t="str"/>
+      <c r="F201" s="12" t="str"/>
       <c r="G201" s="15" t="str"/>
     </row>
     <row r="202">
@@ -2249,8 +2249,8 @@
       <c r="B202" s="12" t="str"/>
       <c r="C202" s="13" t="str"/>
       <c r="D202" s="12" t="str"/>
-      <c r="E202" s="12" t="str"/>
-      <c r="F202" s="14" t="str"/>
+      <c r="E202" s="14" t="str"/>
+      <c r="F202" s="12" t="str"/>
       <c r="G202" s="15" t="str"/>
     </row>
     <row r="203">
@@ -2258,8 +2258,8 @@
       <c r="B203" s="12" t="str"/>
       <c r="C203" s="13" t="str"/>
       <c r="D203" s="12" t="str"/>
-      <c r="E203" s="12" t="str"/>
-      <c r="F203" s="14" t="str"/>
+      <c r="E203" s="14" t="str"/>
+      <c r="F203" s="12" t="str"/>
       <c r="G203" s="15" t="str"/>
     </row>
     <row r="204">
@@ -2267,8 +2267,8 @@
       <c r="B204" s="12" t="str"/>
       <c r="C204" s="13" t="str"/>
       <c r="D204" s="12" t="str"/>
-      <c r="E204" s="12" t="str"/>
-      <c r="F204" s="14" t="str"/>
+      <c r="E204" s="14" t="str"/>
+      <c r="F204" s="12" t="str"/>
       <c r="G204" s="15" t="str"/>
     </row>
     <row r="205">
@@ -2276,8 +2276,8 @@
       <c r="B205" s="12" t="str"/>
       <c r="C205" s="13" t="str"/>
       <c r="D205" s="12" t="str"/>
-      <c r="E205" s="12" t="str"/>
-      <c r="F205" s="14" t="str"/>
+      <c r="E205" s="14" t="str"/>
+      <c r="F205" s="12" t="str"/>
       <c r="G205" s="15" t="str"/>
     </row>
     <row r="206">
@@ -2285,8 +2285,8 @@
       <c r="B206" s="12" t="str"/>
       <c r="C206" s="13" t="str"/>
       <c r="D206" s="12" t="str"/>
-      <c r="E206" s="12" t="str"/>
-      <c r="F206" s="14" t="str"/>
+      <c r="E206" s="14" t="str"/>
+      <c r="F206" s="12" t="str"/>
       <c r="G206" s="15" t="str"/>
     </row>
     <row r="207">
@@ -2294,8 +2294,8 @@
       <c r="B207" s="12" t="str"/>
       <c r="C207" s="13" t="str"/>
       <c r="D207" s="12" t="str"/>
-      <c r="E207" s="12" t="str"/>
-      <c r="F207" s="14" t="str"/>
+      <c r="E207" s="14" t="str"/>
+      <c r="F207" s="12" t="str"/>
       <c r="G207" s="15" t="str"/>
     </row>
     <row r="208">
@@ -2303,8 +2303,8 @@
       <c r="B208" s="12" t="str"/>
       <c r="C208" s="13" t="str"/>
       <c r="D208" s="12" t="str"/>
-      <c r="E208" s="12" t="str"/>
-      <c r="F208" s="14" t="str"/>
+      <c r="E208" s="14" t="str"/>
+      <c r="F208" s="12" t="str"/>
       <c r="G208" s="15" t="str"/>
     </row>
     <row r="209">
@@ -2312,8 +2312,8 @@
       <c r="B209" s="12" t="str"/>
       <c r="C209" s="13" t="str"/>
       <c r="D209" s="12" t="str"/>
-      <c r="E209" s="12" t="str"/>
-      <c r="F209" s="14" t="str"/>
+      <c r="E209" s="14" t="str"/>
+      <c r="F209" s="12" t="str"/>
       <c r="G209" s="15" t="str"/>
     </row>
     <row r="210">
@@ -2321,8 +2321,8 @@
       <c r="B210" s="12" t="str"/>
       <c r="C210" s="13" t="str"/>
       <c r="D210" s="12" t="str"/>
-      <c r="E210" s="12" t="str"/>
-      <c r="F210" s="14" t="str"/>
+      <c r="E210" s="14" t="str"/>
+      <c r="F210" s="12" t="str"/>
       <c r="G210" s="15" t="str"/>
     </row>
     <row r="211">
@@ -2330,8 +2330,8 @@
       <c r="B211" s="12" t="str"/>
       <c r="C211" s="13" t="str"/>
       <c r="D211" s="12" t="str"/>
-      <c r="E211" s="12" t="str"/>
-      <c r="F211" s="14" t="str"/>
+      <c r="E211" s="14" t="str"/>
+      <c r="F211" s="12" t="str"/>
       <c r="G211" s="15" t="str"/>
     </row>
     <row r="212">
@@ -2339,8 +2339,8 @@
       <c r="B212" s="12" t="str"/>
       <c r="C212" s="13" t="str"/>
       <c r="D212" s="12" t="str"/>
-      <c r="E212" s="12" t="str"/>
-      <c r="F212" s="14" t="str"/>
+      <c r="E212" s="14" t="str"/>
+      <c r="F212" s="12" t="str"/>
       <c r="G212" s="15" t="str"/>
     </row>
     <row r="213">
@@ -2348,8 +2348,8 @@
       <c r="B213" s="12" t="str"/>
       <c r="C213" s="13" t="str"/>
       <c r="D213" s="12" t="str"/>
-      <c r="E213" s="12" t="str"/>
-      <c r="F213" s="14" t="str"/>
+      <c r="E213" s="14" t="str"/>
+      <c r="F213" s="12" t="str"/>
       <c r="G213" s="15" t="str"/>
     </row>
     <row r="214">
@@ -2357,8 +2357,8 @@
       <c r="B214" s="12" t="str"/>
       <c r="C214" s="13" t="str"/>
       <c r="D214" s="12" t="str"/>
-      <c r="E214" s="12" t="str"/>
-      <c r="F214" s="14" t="str"/>
+      <c r="E214" s="14" t="str"/>
+      <c r="F214" s="12" t="str"/>
       <c r="G214" s="15" t="str"/>
     </row>
     <row r="215">
@@ -2366,8 +2366,8 @@
       <c r="B215" s="12" t="str"/>
       <c r="C215" s="13" t="str"/>
       <c r="D215" s="12" t="str"/>
-      <c r="E215" s="12" t="str"/>
-      <c r="F215" s="14" t="str"/>
+      <c r="E215" s="14" t="str"/>
+      <c r="F215" s="12" t="str"/>
       <c r="G215" s="15" t="str"/>
     </row>
     <row r="216">
@@ -2375,8 +2375,8 @@
       <c r="B216" s="12" t="str"/>
       <c r="C216" s="13" t="str"/>
       <c r="D216" s="12" t="str"/>
-      <c r="E216" s="12" t="str"/>
-      <c r="F216" s="14" t="str"/>
+      <c r="E216" s="14" t="str"/>
+      <c r="F216" s="12" t="str"/>
       <c r="G216" s="15" t="str"/>
     </row>
     <row r="217">
@@ -2384,8 +2384,8 @@
       <c r="B217" s="12" t="str"/>
       <c r="C217" s="13" t="str"/>
       <c r="D217" s="12" t="str"/>
-      <c r="E217" s="12" t="str"/>
-      <c r="F217" s="14" t="str"/>
+      <c r="E217" s="14" t="str"/>
+      <c r="F217" s="12" t="str"/>
       <c r="G217" s="15" t="str"/>
     </row>
     <row r="218">
@@ -2393,8 +2393,8 @@
       <c r="B218" s="12" t="str"/>
       <c r="C218" s="13" t="str"/>
       <c r="D218" s="12" t="str"/>
-      <c r="E218" s="12" t="str"/>
-      <c r="F218" s="14" t="str"/>
+      <c r="E218" s="14" t="str"/>
+      <c r="F218" s="12" t="str"/>
       <c r="G218" s="15" t="str"/>
     </row>
     <row r="219">
@@ -2402,8 +2402,8 @@
       <c r="B219" s="12" t="str"/>
       <c r="C219" s="13" t="str"/>
       <c r="D219" s="12" t="str"/>
-      <c r="E219" s="12" t="str"/>
-      <c r="F219" s="14" t="str"/>
+      <c r="E219" s="14" t="str"/>
+      <c r="F219" s="12" t="str"/>
       <c r="G219" s="15" t="str"/>
     </row>
     <row r="220">
@@ -2411,8 +2411,8 @@
       <c r="B220" s="12" t="str"/>
       <c r="C220" s="13" t="str"/>
       <c r="D220" s="12" t="str"/>
-      <c r="E220" s="12" t="str"/>
-      <c r="F220" s="14" t="str"/>
+      <c r="E220" s="14" t="str"/>
+      <c r="F220" s="12" t="str"/>
       <c r="G220" s="15" t="str"/>
     </row>
     <row r="221">
@@ -2420,8 +2420,8 @@
       <c r="B221" s="12" t="str"/>
       <c r="C221" s="13" t="str"/>
       <c r="D221" s="12" t="str"/>
-      <c r="E221" s="12" t="str"/>
-      <c r="F221" s="14" t="str"/>
+      <c r="E221" s="14" t="str"/>
+      <c r="F221" s="12" t="str"/>
       <c r="G221" s="15" t="str"/>
     </row>
     <row r="222">
@@ -2429,8 +2429,8 @@
       <c r="B222" s="12" t="str"/>
       <c r="C222" s="13" t="str"/>
       <c r="D222" s="12" t="str"/>
-      <c r="E222" s="12" t="str"/>
-      <c r="F222" s="14" t="str"/>
+      <c r="E222" s="14" t="str"/>
+      <c r="F222" s="12" t="str"/>
       <c r="G222" s="15" t="str"/>
     </row>
     <row r="223">
@@ -2438,8 +2438,8 @@
       <c r="B223" s="12" t="str"/>
       <c r="C223" s="13" t="str"/>
       <c r="D223" s="12" t="str"/>
-      <c r="E223" s="12" t="str"/>
-      <c r="F223" s="14" t="str"/>
+      <c r="E223" s="14" t="str"/>
+      <c r="F223" s="12" t="str"/>
       <c r="G223" s="15" t="str"/>
     </row>
     <row r="224">
@@ -2447,8 +2447,8 @@
       <c r="B224" s="12" t="str"/>
       <c r="C224" s="13" t="str"/>
       <c r="D224" s="12" t="str"/>
-      <c r="E224" s="12" t="str"/>
-      <c r="F224" s="14" t="str"/>
+      <c r="E224" s="14" t="str"/>
+      <c r="F224" s="12" t="str"/>
       <c r="G224" s="15" t="str"/>
     </row>
     <row r="225">
@@ -2456,8 +2456,8 @@
       <c r="B225" s="12" t="str"/>
       <c r="C225" s="13" t="str"/>
       <c r="D225" s="12" t="str"/>
-      <c r="E225" s="12" t="str"/>
-      <c r="F225" s="14" t="str"/>
+      <c r="E225" s="14" t="str"/>
+      <c r="F225" s="12" t="str"/>
       <c r="G225" s="15" t="str"/>
     </row>
     <row r="226">
@@ -2465,8 +2465,8 @@
       <c r="B226" s="12" t="str"/>
       <c r="C226" s="13" t="str"/>
       <c r="D226" s="12" t="str"/>
-      <c r="E226" s="12" t="str"/>
-      <c r="F226" s="14" t="str"/>
+      <c r="E226" s="14" t="str"/>
+      <c r="F226" s="12" t="str"/>
       <c r="G226" s="15" t="str"/>
     </row>
     <row r="227">
@@ -2474,8 +2474,8 @@
       <c r="B227" s="12" t="str"/>
       <c r="C227" s="13" t="str"/>
       <c r="D227" s="12" t="str"/>
-      <c r="E227" s="12" t="str"/>
-      <c r="F227" s="14" t="str"/>
+      <c r="E227" s="14" t="str"/>
+      <c r="F227" s="12" t="str"/>
       <c r="G227" s="15" t="str"/>
     </row>
     <row r="228">
@@ -2483,8 +2483,8 @@
       <c r="B228" s="12" t="str"/>
       <c r="C228" s="13" t="str"/>
       <c r="D228" s="12" t="str"/>
-      <c r="E228" s="12" t="str"/>
-      <c r="F228" s="14" t="str"/>
+      <c r="E228" s="14" t="str"/>
+      <c r="F228" s="12" t="str"/>
       <c r="G228" s="15" t="str"/>
     </row>
     <row r="229">
@@ -2492,8 +2492,8 @@
       <c r="B229" s="12" t="str"/>
       <c r="C229" s="13" t="str"/>
       <c r="D229" s="12" t="str"/>
-      <c r="E229" s="12" t="str"/>
-      <c r="F229" s="14" t="str"/>
+      <c r="E229" s="14" t="str"/>
+      <c r="F229" s="12" t="str"/>
       <c r="G229" s="15" t="str"/>
     </row>
     <row r="230">
@@ -2501,8 +2501,8 @@
       <c r="B230" s="12" t="str"/>
       <c r="C230" s="13" t="str"/>
       <c r="D230" s="12" t="str"/>
-      <c r="E230" s="12" t="str"/>
-      <c r="F230" s="14" t="str"/>
+      <c r="E230" s="14" t="str"/>
+      <c r="F230" s="12" t="str"/>
       <c r="G230" s="15" t="str"/>
     </row>
     <row r="231">
@@ -2510,8 +2510,8 @@
       <c r="B231" s="12" t="str"/>
       <c r="C231" s="13" t="str"/>
       <c r="D231" s="12" t="str"/>
-      <c r="E231" s="12" t="str"/>
-      <c r="F231" s="14" t="str"/>
+      <c r="E231" s="14" t="str"/>
+      <c r="F231" s="12" t="str"/>
       <c r="G231" s="15" t="str"/>
     </row>
     <row r="232">
@@ -2519,8 +2519,8 @@
       <c r="B232" s="12" t="str"/>
       <c r="C232" s="13" t="str"/>
       <c r="D232" s="12" t="str"/>
-      <c r="E232" s="12" t="str"/>
-      <c r="F232" s="14" t="str"/>
+      <c r="E232" s="14" t="str"/>
+      <c r="F232" s="12" t="str"/>
       <c r="G232" s="15" t="str"/>
     </row>
     <row r="233">
@@ -2528,8 +2528,8 @@
       <c r="B233" s="12" t="str"/>
       <c r="C233" s="13" t="str"/>
       <c r="D233" s="12" t="str"/>
-      <c r="E233" s="12" t="str"/>
-      <c r="F233" s="14" t="str"/>
+      <c r="E233" s="14" t="str"/>
+      <c r="F233" s="12" t="str"/>
       <c r="G233" s="15" t="str"/>
     </row>
     <row r="234">
@@ -2537,8 +2537,8 @@
       <c r="B234" s="12" t="str"/>
       <c r="C234" s="13" t="str"/>
       <c r="D234" s="12" t="str"/>
-      <c r="E234" s="12" t="str"/>
-      <c r="F234" s="14" t="str"/>
+      <c r="E234" s="14" t="str"/>
+      <c r="F234" s="12" t="str"/>
       <c r="G234" s="15" t="str"/>
     </row>
     <row r="235">
@@ -2546,8 +2546,8 @@
       <c r="B235" s="12" t="str"/>
       <c r="C235" s="13" t="str"/>
       <c r="D235" s="12" t="str"/>
-      <c r="E235" s="12" t="str"/>
-      <c r="F235" s="14" t="str"/>
+      <c r="E235" s="14" t="str"/>
+      <c r="F235" s="12" t="str"/>
       <c r="G235" s="15" t="str"/>
     </row>
     <row r="236">
@@ -2555,8 +2555,8 @@
       <c r="B236" s="12" t="str"/>
       <c r="C236" s="13" t="str"/>
       <c r="D236" s="12" t="str"/>
-      <c r="E236" s="12" t="str"/>
-      <c r="F236" s="14" t="str"/>
+      <c r="E236" s="14" t="str"/>
+      <c r="F236" s="12" t="str"/>
       <c r="G236" s="15" t="str"/>
     </row>
     <row r="237">
@@ -2564,8 +2564,8 @@
       <c r="B237" s="12" t="str"/>
       <c r="C237" s="13" t="str"/>
       <c r="D237" s="12" t="str"/>
-      <c r="E237" s="12" t="str"/>
-      <c r="F237" s="14" t="str"/>
+      <c r="E237" s="14" t="str"/>
+      <c r="F237" s="12" t="str"/>
       <c r="G237" s="15" t="str"/>
     </row>
     <row r="238">
@@ -2573,8 +2573,8 @@
       <c r="B238" s="12" t="str"/>
       <c r="C238" s="13" t="str"/>
       <c r="D238" s="12" t="str"/>
-      <c r="E238" s="12" t="str"/>
-      <c r="F238" s="14" t="str"/>
+      <c r="E238" s="14" t="str"/>
+      <c r="F238" s="12" t="str"/>
       <c r="G238" s="15" t="str"/>
     </row>
     <row r="239">
@@ -2582,8 +2582,8 @@
       <c r="B239" s="12" t="str"/>
       <c r="C239" s="13" t="str"/>
       <c r="D239" s="12" t="str"/>
-      <c r="E239" s="12" t="str"/>
-      <c r="F239" s="14" t="str"/>
+      <c r="E239" s="14" t="str"/>
+      <c r="F239" s="12" t="str"/>
       <c r="G239" s="15" t="str"/>
     </row>
     <row r="240">
@@ -2591,8 +2591,8 @@
       <c r="B240" s="12" t="str"/>
       <c r="C240" s="13" t="str"/>
       <c r="D240" s="12" t="str"/>
-      <c r="E240" s="12" t="str"/>
-      <c r="F240" s="14" t="str"/>
+      <c r="E240" s="14" t="str"/>
+      <c r="F240" s="12" t="str"/>
       <c r="G240" s="15" t="str"/>
     </row>
     <row r="241">
@@ -2600,8 +2600,8 @@
       <c r="B241" s="12" t="str"/>
       <c r="C241" s="13" t="str"/>
       <c r="D241" s="12" t="str"/>
-      <c r="E241" s="12" t="str"/>
-      <c r="F241" s="14" t="str"/>
+      <c r="E241" s="14" t="str"/>
+      <c r="F241" s="12" t="str"/>
       <c r="G241" s="15" t="str"/>
     </row>
     <row r="242">
@@ -2609,8 +2609,8 @@
       <c r="B242" s="12" t="str"/>
       <c r="C242" s="13" t="str"/>
       <c r="D242" s="12" t="str"/>
-      <c r="E242" s="12" t="str"/>
-      <c r="F242" s="14" t="str"/>
+      <c r="E242" s="14" t="str"/>
+      <c r="F242" s="12" t="str"/>
       <c r="G242" s="15" t="str"/>
     </row>
     <row r="243">
@@ -2618,8 +2618,8 @@
       <c r="B243" s="12" t="str"/>
       <c r="C243" s="13" t="str"/>
       <c r="D243" s="12" t="str"/>
-      <c r="E243" s="12" t="str"/>
-      <c r="F243" s="14" t="str"/>
+      <c r="E243" s="14" t="str"/>
+      <c r="F243" s="12" t="str"/>
       <c r="G243" s="15" t="str"/>
     </row>
     <row r="244">
@@ -2627,8 +2627,8 @@
       <c r="B244" s="12" t="str"/>
       <c r="C244" s="13" t="str"/>
       <c r="D244" s="12" t="str"/>
-      <c r="E244" s="12" t="str"/>
-      <c r="F244" s="14" t="str"/>
+      <c r="E244" s="14" t="str"/>
+      <c r="F244" s="12" t="str"/>
       <c r="G244" s="15" t="str"/>
     </row>
     <row r="245">
@@ -2636,8 +2636,8 @@
       <c r="B245" s="12" t="str"/>
       <c r="C245" s="13" t="str"/>
       <c r="D245" s="12" t="str"/>
-      <c r="E245" s="12" t="str"/>
-      <c r="F245" s="14" t="str"/>
+      <c r="E245" s="14" t="str"/>
+      <c r="F245" s="12" t="str"/>
       <c r="G245" s="15" t="str"/>
     </row>
     <row r="246">
@@ -2645,8 +2645,8 @@
       <c r="B246" s="12" t="str"/>
       <c r="C246" s="13" t="str"/>
       <c r="D246" s="12" t="str"/>
-      <c r="E246" s="12" t="str"/>
-      <c r="F246" s="14" t="str"/>
+      <c r="E246" s="14" t="str"/>
+      <c r="F246" s="12" t="str"/>
       <c r="G246" s="15" t="str"/>
     </row>
     <row r="247">
@@ -2654,8 +2654,8 @@
       <c r="B247" s="12" t="str"/>
       <c r="C247" s="13" t="str"/>
       <c r="D247" s="12" t="str"/>
-      <c r="E247" s="12" t="str"/>
-      <c r="F247" s="14" t="str"/>
+      <c r="E247" s="14" t="str"/>
+      <c r="F247" s="12" t="str"/>
       <c r="G247" s="15" t="str"/>
     </row>
     <row r="248">
@@ -2663,8 +2663,8 @@
       <c r="B248" s="12" t="str"/>
       <c r="C248" s="13" t="str"/>
       <c r="D248" s="12" t="str"/>
-      <c r="E248" s="12" t="str"/>
-      <c r="F248" s="14" t="str"/>
+      <c r="E248" s="14" t="str"/>
+      <c r="F248" s="12" t="str"/>
       <c r="G248" s="15" t="str"/>
     </row>
     <row r="249">
@@ -2672,8 +2672,8 @@
       <c r="B249" s="12" t="str"/>
       <c r="C249" s="13" t="str"/>
       <c r="D249" s="12" t="str"/>
-      <c r="E249" s="12" t="str"/>
-      <c r="F249" s="14" t="str"/>
+      <c r="E249" s="14" t="str"/>
+      <c r="F249" s="12" t="str"/>
       <c r="G249" s="15" t="str"/>
     </row>
     <row r="250">
@@ -2681,8 +2681,8 @@
       <c r="B250" s="12" t="str"/>
       <c r="C250" s="13" t="str"/>
       <c r="D250" s="12" t="str"/>
-      <c r="E250" s="12" t="str"/>
-      <c r="F250" s="14" t="str"/>
+      <c r="E250" s="14" t="str"/>
+      <c r="F250" s="12" t="str"/>
       <c r="G250" s="15" t="str"/>
     </row>
     <row r="251">
@@ -2690,8 +2690,8 @@
       <c r="B251" s="12" t="str"/>
       <c r="C251" s="13" t="str"/>
       <c r="D251" s="12" t="str"/>
-      <c r="E251" s="12" t="str"/>
-      <c r="F251" s="14" t="str"/>
+      <c r="E251" s="14" t="str"/>
+      <c r="F251" s="12" t="str"/>
       <c r="G251" s="15" t="str"/>
     </row>
     <row r="252">
@@ -2699,8 +2699,8 @@
       <c r="B252" s="12" t="str"/>
       <c r="C252" s="13" t="str"/>
       <c r="D252" s="12" t="str"/>
-      <c r="E252" s="12" t="str"/>
-      <c r="F252" s="14" t="str"/>
+      <c r="E252" s="14" t="str"/>
+      <c r="F252" s="12" t="str"/>
       <c r="G252" s="15" t="str"/>
     </row>
     <row r="253">
@@ -2708,8 +2708,8 @@
       <c r="B253" s="12" t="str"/>
       <c r="C253" s="13" t="str"/>
       <c r="D253" s="12" t="str"/>
-      <c r="E253" s="12" t="str"/>
-      <c r="F253" s="14" t="str"/>
+      <c r="E253" s="14" t="str"/>
+      <c r="F253" s="12" t="str"/>
       <c r="G253" s="15" t="str"/>
     </row>
     <row r="254">
@@ -2717,8 +2717,8 @@
       <c r="B254" s="12" t="str"/>
       <c r="C254" s="13" t="str"/>
       <c r="D254" s="12" t="str"/>
-      <c r="E254" s="12" t="str"/>
-      <c r="F254" s="14" t="str"/>
+      <c r="E254" s="14" t="str"/>
+      <c r="F254" s="12" t="str"/>
       <c r="G254" s="15" t="str"/>
     </row>
     <row r="255">
@@ -2726,8 +2726,8 @@
       <c r="B255" s="12" t="str"/>
       <c r="C255" s="13" t="str"/>
       <c r="D255" s="12" t="str"/>
-      <c r="E255" s="12" t="str"/>
-      <c r="F255" s="14" t="str"/>
+      <c r="E255" s="14" t="str"/>
+      <c r="F255" s="12" t="str"/>
       <c r="G255" s="15" t="str"/>
     </row>
     <row r="256">
@@ -2735,8 +2735,8 @@
       <c r="B256" s="12" t="str"/>
       <c r="C256" s="13" t="str"/>
       <c r="D256" s="12" t="str"/>
-      <c r="E256" s="12" t="str"/>
-      <c r="F256" s="14" t="str"/>
+      <c r="E256" s="14" t="str"/>
+      <c r="F256" s="12" t="str"/>
       <c r="G256" s="15" t="str"/>
     </row>
     <row r="257">
@@ -2744,8 +2744,8 @@
       <c r="B257" s="12" t="str"/>
       <c r="C257" s="13" t="str"/>
       <c r="D257" s="12" t="str"/>
-      <c r="E257" s="12" t="str"/>
-      <c r="F257" s="14" t="str"/>
+      <c r="E257" s="14" t="str"/>
+      <c r="F257" s="12" t="str"/>
       <c r="G257" s="15" t="str"/>
     </row>
     <row r="258">
@@ -2753,8 +2753,8 @@
       <c r="B258" s="12" t="str"/>
       <c r="C258" s="13" t="str"/>
       <c r="D258" s="12" t="str"/>
-      <c r="E258" s="12" t="str"/>
-      <c r="F258" s="14" t="str"/>
+      <c r="E258" s="14" t="str"/>
+      <c r="F258" s="12" t="str"/>
       <c r="G258" s="15" t="str"/>
     </row>
     <row r="259">
@@ -2762,8 +2762,8 @@
       <c r="B259" s="12" t="str"/>
       <c r="C259" s="13" t="str"/>
       <c r="D259" s="12" t="str"/>
-      <c r="E259" s="12" t="str"/>
-      <c r="F259" s="14" t="str"/>
+      <c r="E259" s="14" t="str"/>
+      <c r="F259" s="12" t="str"/>
       <c r="G259" s="15" t="str"/>
     </row>
     <row r="260">
@@ -2771,8 +2771,8 @@
       <c r="B260" s="12" t="str"/>
       <c r="C260" s="13" t="str"/>
       <c r="D260" s="12" t="str"/>
-      <c r="E260" s="12" t="str"/>
-      <c r="F260" s="14" t="str"/>
+      <c r="E260" s="14" t="str"/>
+      <c r="F260" s="12" t="str"/>
       <c r="G260" s="15" t="str"/>
     </row>
     <row r="261">
@@ -2780,8 +2780,8 @@
       <c r="B261" s="12" t="str"/>
       <c r="C261" s="13" t="str"/>
       <c r="D261" s="12" t="str"/>
-      <c r="E261" s="12" t="str"/>
-      <c r="F261" s="14" t="str"/>
+      <c r="E261" s="14" t="str"/>
+      <c r="F261" s="12" t="str"/>
       <c r="G261" s="15" t="str"/>
     </row>
     <row r="262">
@@ -2789,8 +2789,8 @@
       <c r="B262" s="12" t="str"/>
       <c r="C262" s="13" t="str"/>
       <c r="D262" s="12" t="str"/>
-      <c r="E262" s="12" t="str"/>
-      <c r="F262" s="14" t="str"/>
+      <c r="E262" s="14" t="str"/>
+      <c r="F262" s="12" t="str"/>
       <c r="G262" s="15" t="str"/>
     </row>
     <row r="263">
@@ -2798,8 +2798,8 @@
       <c r="B263" s="12" t="str"/>
       <c r="C263" s="13" t="str"/>
       <c r="D263" s="12" t="str"/>
-      <c r="E263" s="12" t="str"/>
-      <c r="F263" s="14" t="str"/>
+      <c r="E263" s="14" t="str"/>
+      <c r="F263" s="12" t="str"/>
       <c r="G263" s="15" t="str"/>
     </row>
     <row r="264">
@@ -2807,8 +2807,8 @@
       <c r="B264" s="12" t="str"/>
       <c r="C264" s="13" t="str"/>
       <c r="D264" s="12" t="str"/>
-      <c r="E264" s="12" t="str"/>
-      <c r="F264" s="14" t="str"/>
+      <c r="E264" s="14" t="str"/>
+      <c r="F264" s="12" t="str"/>
       <c r="G264" s="15" t="str"/>
     </row>
     <row r="265">
@@ -2816,8 +2816,8 @@
       <c r="B265" s="12" t="str"/>
       <c r="C265" s="13" t="str"/>
       <c r="D265" s="12" t="str"/>
-      <c r="E265" s="12" t="str"/>
-      <c r="F265" s="14" t="str"/>
+      <c r="E265" s="14" t="str"/>
+      <c r="F265" s="12" t="str"/>
       <c r="G265" s="15" t="str"/>
     </row>
     <row r="266">
@@ -2825,8 +2825,8 @@
       <c r="B266" s="12" t="str"/>
       <c r="C266" s="13" t="str"/>
       <c r="D266" s="12" t="str"/>
-      <c r="E266" s="12" t="str"/>
-      <c r="F266" s="14" t="str"/>
+      <c r="E266" s="14" t="str"/>
+      <c r="F266" s="12" t="str"/>
       <c r="G266" s="15" t="str"/>
     </row>
     <row r="267">
@@ -2834,8 +2834,8 @@
       <c r="B267" s="12" t="str"/>
       <c r="C267" s="13" t="str"/>
       <c r="D267" s="12" t="str"/>
-      <c r="E267" s="12" t="str"/>
-      <c r="F267" s="14" t="str"/>
+      <c r="E267" s="14" t="str"/>
+      <c r="F267" s="12" t="str"/>
       <c r="G267" s="15" t="str"/>
     </row>
     <row r="268">
@@ -2843,8 +2843,8 @@
       <c r="B268" s="12" t="str"/>
       <c r="C268" s="13" t="str"/>
       <c r="D268" s="12" t="str"/>
-      <c r="E268" s="12" t="str"/>
-      <c r="F268" s="14" t="str"/>
+      <c r="E268" s="14" t="str"/>
+      <c r="F268" s="12" t="str"/>
       <c r="G268" s="15" t="str"/>
     </row>
     <row r="269">
@@ -2852,8 +2852,8 @@
       <c r="B269" s="12" t="str"/>
       <c r="C269" s="13" t="str"/>
       <c r="D269" s="12" t="str"/>
-      <c r="E269" s="12" t="str"/>
-      <c r="F269" s="14" t="str"/>
+      <c r="E269" s="14" t="str"/>
+      <c r="F269" s="12" t="str"/>
       <c r="G269" s="15" t="str"/>
     </row>
     <row r="270">
@@ -2861,8 +2861,8 @@
       <c r="B270" s="12" t="str"/>
       <c r="C270" s="13" t="str"/>
       <c r="D270" s="12" t="str"/>
-      <c r="E270" s="12" t="str"/>
-      <c r="F270" s="14" t="str"/>
+      <c r="E270" s="14" t="str"/>
+      <c r="F270" s="12" t="str"/>
       <c r="G270" s="15" t="str"/>
     </row>
     <row r="271">
@@ -2870,8 +2870,8 @@
       <c r="B271" s="12" t="str"/>
       <c r="C271" s="13" t="str"/>
       <c r="D271" s="12" t="str"/>
-      <c r="E271" s="12" t="str"/>
-      <c r="F271" s="14" t="str"/>
+      <c r="E271" s="14" t="str"/>
+      <c r="F271" s="12" t="str"/>
       <c r="G271" s="15" t="str"/>
     </row>
     <row r="272">
@@ -2879,8 +2879,8 @@
       <c r="B272" s="12" t="str"/>
       <c r="C272" s="13" t="str"/>
       <c r="D272" s="12" t="str"/>
-      <c r="E272" s="12" t="str"/>
-      <c r="F272" s="14" t="str"/>
+      <c r="E272" s="14" t="str"/>
+      <c r="F272" s="12" t="str"/>
       <c r="G272" s="15" t="str"/>
     </row>
     <row r="273">
@@ -2888,8 +2888,8 @@
       <c r="B273" s="12" t="str"/>
       <c r="C273" s="13" t="str"/>
       <c r="D273" s="12" t="str"/>
-      <c r="E273" s="12" t="str"/>
-      <c r="F273" s="14" t="str"/>
+      <c r="E273" s="14" t="str"/>
+      <c r="F273" s="12" t="str"/>
       <c r="G273" s="15" t="str"/>
     </row>
     <row r="274">
@@ -2897,8 +2897,8 @@
       <c r="B274" s="12" t="str"/>
       <c r="C274" s="13" t="str"/>
       <c r="D274" s="12" t="str"/>
-      <c r="E274" s="12" t="str"/>
-      <c r="F274" s="14" t="str"/>
+      <c r="E274" s="14" t="str"/>
+      <c r="F274" s="12" t="str"/>
       <c r="G274" s="15" t="str"/>
     </row>
     <row r="275">
@@ -2906,8 +2906,8 @@
       <c r="B275" s="12" t="str"/>
       <c r="C275" s="13" t="str"/>
       <c r="D275" s="12" t="str"/>
-      <c r="E275" s="12" t="str"/>
-      <c r="F275" s="14" t="str"/>
+      <c r="E275" s="14" t="str"/>
+      <c r="F275" s="12" t="str"/>
       <c r="G275" s="15" t="str"/>
     </row>
     <row r="276">
@@ -2915,8 +2915,8 @@
       <c r="B276" s="12" t="str"/>
       <c r="C276" s="13" t="str"/>
       <c r="D276" s="12" t="str"/>
-      <c r="E276" s="12" t="str"/>
-      <c r="F276" s="14" t="str"/>
+      <c r="E276" s="14" t="str"/>
+      <c r="F276" s="12" t="str"/>
       <c r="G276" s="15" t="str"/>
     </row>
     <row r="277">
@@ -2924,8 +2924,8 @@
       <c r="B277" s="12" t="str"/>
       <c r="C277" s="13" t="str"/>
       <c r="D277" s="12" t="str"/>
-      <c r="E277" s="12" t="str"/>
-      <c r="F277" s="14" t="str"/>
+      <c r="E277" s="14" t="str"/>
+      <c r="F277" s="12" t="str"/>
       <c r="G277" s="15" t="str"/>
     </row>
     <row r="278">
@@ -2933,8 +2933,8 @@
       <c r="B278" s="12" t="str"/>
       <c r="C278" s="13" t="str"/>
       <c r="D278" s="12" t="str"/>
-      <c r="E278" s="12" t="str"/>
-      <c r="F278" s="14" t="str"/>
+      <c r="E278" s="14" t="str"/>
+      <c r="F278" s="12" t="str"/>
       <c r="G278" s="15" t="str"/>
     </row>
     <row r="279">
@@ -2942,8 +2942,8 @@
       <c r="B279" s="12" t="str"/>
       <c r="C279" s="13" t="str"/>
       <c r="D279" s="12" t="str"/>
-      <c r="E279" s="12" t="str"/>
-      <c r="F279" s="14" t="str"/>
+      <c r="E279" s="14" t="str"/>
+      <c r="F279" s="12" t="str"/>
       <c r="G279" s="15" t="str"/>
     </row>
     <row r="280">
@@ -2951,8 +2951,8 @@
       <c r="B280" s="12" t="str"/>
       <c r="C280" s="13" t="str"/>
       <c r="D280" s="12" t="str"/>
-      <c r="E280" s="12" t="str"/>
-      <c r="F280" s="14" t="str"/>
+      <c r="E280" s="14" t="str"/>
+      <c r="F280" s="12" t="str"/>
       <c r="G280" s="15" t="str"/>
     </row>
     <row r="281">
@@ -2960,8 +2960,8 @@
       <c r="B281" s="12" t="str"/>
       <c r="C281" s="13" t="str"/>
       <c r="D281" s="12" t="str"/>
-      <c r="E281" s="12" t="str"/>
-      <c r="F281" s="14" t="str"/>
+      <c r="E281" s="14" t="str"/>
+      <c r="F281" s="12" t="str"/>
       <c r="G281" s="15" t="str"/>
     </row>
     <row r="282">
@@ -2969,8 +2969,8 @@
       <c r="B282" s="12" t="str"/>
       <c r="C282" s="13" t="str"/>
       <c r="D282" s="12" t="str"/>
-      <c r="E282" s="12" t="str"/>
-      <c r="F282" s="14" t="str"/>
+      <c r="E282" s="14" t="str"/>
+      <c r="F282" s="12" t="str"/>
       <c r="G282" s="15" t="str"/>
     </row>
     <row r="283">
@@ -2978,8 +2978,8 @@
       <c r="B283" s="12" t="str"/>
       <c r="C283" s="13" t="str"/>
       <c r="D283" s="12" t="str"/>
-      <c r="E283" s="12" t="str"/>
-      <c r="F283" s="14" t="str"/>
+      <c r="E283" s="14" t="str"/>
+      <c r="F283" s="12" t="str"/>
       <c r="G283" s="15" t="str"/>
     </row>
     <row r="284">
@@ -2987,8 +2987,8 @@
       <c r="B284" s="12" t="str"/>
       <c r="C284" s="13" t="str"/>
       <c r="D284" s="12" t="str"/>
-      <c r="E284" s="12" t="str"/>
-      <c r="F284" s="14" t="str"/>
+      <c r="E284" s="14" t="str"/>
+      <c r="F284" s="12" t="str"/>
       <c r="G284" s="15" t="str"/>
     </row>
     <row r="285">
@@ -2996,8 +2996,8 @@
       <c r="B285" s="12" t="str"/>
       <c r="C285" s="13" t="str"/>
       <c r="D285" s="12" t="str"/>
-      <c r="E285" s="12" t="str"/>
-      <c r="F285" s="14" t="str"/>
+      <c r="E285" s="14" t="str"/>
+      <c r="F285" s="12" t="str"/>
       <c r="G285" s="15" t="str"/>
     </row>
     <row r="286">
@@ -3005,8 +3005,8 @@
       <c r="B286" s="12" t="str"/>
       <c r="C286" s="13" t="str"/>
       <c r="D286" s="12" t="str"/>
-      <c r="E286" s="12" t="str"/>
-      <c r="F286" s="14" t="str"/>
+      <c r="E286" s="14" t="str"/>
+      <c r="F286" s="12" t="str"/>
       <c r="G286" s="15" t="str"/>
     </row>
     <row r="287">
@@ -3014,8 +3014,8 @@
       <c r="B287" s="12" t="str"/>
       <c r="C287" s="13" t="str"/>
       <c r="D287" s="12" t="str"/>
-      <c r="E287" s="12" t="str"/>
-      <c r="F287" s="14" t="str"/>
+      <c r="E287" s="14" t="str"/>
+      <c r="F287" s="12" t="str"/>
       <c r="G287" s="15" t="str"/>
     </row>
     <row r="288">
@@ -3023,8 +3023,8 @@
       <c r="B288" s="12" t="str"/>
       <c r="C288" s="13" t="str"/>
       <c r="D288" s="12" t="str"/>
-      <c r="E288" s="12" t="str"/>
-      <c r="F288" s="14" t="str"/>
+      <c r="E288" s="14" t="str"/>
+      <c r="F288" s="12" t="str"/>
       <c r="G288" s="15" t="str"/>
     </row>
     <row r="289">
@@ -3032,8 +3032,8 @@
       <c r="B289" s="12" t="str"/>
       <c r="C289" s="13" t="str"/>
       <c r="D289" s="12" t="str"/>
-      <c r="E289" s="12" t="str"/>
-      <c r="F289" s="14" t="str"/>
+      <c r="E289" s="14" t="str"/>
+      <c r="F289" s="12" t="str"/>
       <c r="G289" s="15" t="str"/>
     </row>
     <row r="290">
@@ -3041,8 +3041,8 @@
       <c r="B290" s="12" t="str"/>
       <c r="C290" s="13" t="str"/>
       <c r="D290" s="12" t="str"/>
-      <c r="E290" s="12" t="str"/>
-      <c r="F290" s="14" t="str"/>
+      <c r="E290" s="14" t="str"/>
+      <c r="F290" s="12" t="str"/>
       <c r="G290" s="15" t="str"/>
     </row>
     <row r="291">
@@ -3050,8 +3050,8 @@
       <c r="B291" s="12" t="str"/>
       <c r="C291" s="13" t="str"/>
       <c r="D291" s="12" t="str"/>
-      <c r="E291" s="12" t="str"/>
-      <c r="F291" s="14" t="str"/>
+      <c r="E291" s="14" t="str"/>
+      <c r="F291" s="12" t="str"/>
       <c r="G291" s="15" t="str"/>
     </row>
     <row r="292">
@@ -3059,8 +3059,8 @@
       <c r="B292" s="12" t="str"/>
       <c r="C292" s="13" t="str"/>
       <c r="D292" s="12" t="str"/>
-      <c r="E292" s="12" t="str"/>
-      <c r="F292" s="14" t="str"/>
+      <c r="E292" s="14" t="str"/>
+      <c r="F292" s="12" t="str"/>
       <c r="G292" s="15" t="str"/>
     </row>
     <row r="293">
@@ -3068,8 +3068,8 @@
       <c r="B293" s="12" t="str"/>
       <c r="C293" s="13" t="str"/>
       <c r="D293" s="12" t="str"/>
-      <c r="E293" s="12" t="str"/>
-      <c r="F293" s="14" t="str"/>
+      <c r="E293" s="14" t="str"/>
+      <c r="F293" s="12" t="str"/>
       <c r="G293" s="15" t="str"/>
     </row>
     <row r="294">
@@ -3077,8 +3077,8 @@
       <c r="B294" s="12" t="str"/>
       <c r="C294" s="13" t="str"/>
       <c r="D294" s="12" t="str"/>
-      <c r="E294" s="12" t="str"/>
-      <c r="F294" s="14" t="str"/>
+      <c r="E294" s="14" t="str"/>
+      <c r="F294" s="12" t="str"/>
       <c r="G294" s="15" t="str"/>
     </row>
     <row r="295">
@@ -3086,8 +3086,8 @@
       <c r="B295" s="12" t="str"/>
       <c r="C295" s="13" t="str"/>
       <c r="D295" s="12" t="str"/>
-      <c r="E295" s="12" t="str"/>
-      <c r="F295" s="14" t="str"/>
+      <c r="E295" s="14" t="str"/>
+      <c r="F295" s="12" t="str"/>
       <c r="G295" s="15" t="str"/>
     </row>
     <row r="296">
@@ -3095,8 +3095,8 @@
       <c r="B296" s="12" t="str"/>
       <c r="C296" s="13" t="str"/>
       <c r="D296" s="12" t="str"/>
-      <c r="E296" s="12" t="str"/>
-      <c r="F296" s="14" t="str"/>
+      <c r="E296" s="14" t="str"/>
+      <c r="F296" s="12" t="str"/>
       <c r="G296" s="15" t="str"/>
     </row>
     <row r="297">
@@ -3104,8 +3104,8 @@
       <c r="B297" s="12" t="str"/>
       <c r="C297" s="13" t="str"/>
       <c r="D297" s="12" t="str"/>
-      <c r="E297" s="12" t="str"/>
-      <c r="F297" s="14" t="str"/>
+      <c r="E297" s="14" t="str"/>
+      <c r="F297" s="12" t="str"/>
       <c r="G297" s="15" t="str"/>
     </row>
     <row r="298">
@@ -3113,8 +3113,8 @@
       <c r="B298" s="12" t="str"/>
       <c r="C298" s="13" t="str"/>
       <c r="D298" s="12" t="str"/>
-      <c r="E298" s="12" t="str"/>
-      <c r="F298" s="14" t="str"/>
+      <c r="E298" s="14" t="str"/>
+      <c r="F298" s="12" t="str"/>
       <c r="G298" s="15" t="str"/>
     </row>
     <row r="299">
@@ -3122,8 +3122,8 @@
       <c r="B299" s="12" t="str"/>
       <c r="C299" s="13" t="str"/>
       <c r="D299" s="12" t="str"/>
-      <c r="E299" s="12" t="str"/>
-      <c r="F299" s="14" t="str"/>
+      <c r="E299" s="14" t="str"/>
+      <c r="F299" s="12" t="str"/>
       <c r="G299" s="15" t="str"/>
     </row>
     <row r="300">
@@ -3131,8 +3131,8 @@
       <c r="B300" s="12" t="str"/>
       <c r="C300" s="13" t="str"/>
       <c r="D300" s="12" t="str"/>
-      <c r="E300" s="12" t="str"/>
-      <c r="F300" s="14" t="str"/>
+      <c r="E300" s="14" t="str"/>
+      <c r="F300" s="12" t="str"/>
       <c r="G300" s="15" t="str"/>
     </row>
     <row r="301">
@@ -3140,8 +3140,8 @@
       <c r="B301" s="12" t="str"/>
       <c r="C301" s="13" t="str"/>
       <c r="D301" s="12" t="str"/>
-      <c r="E301" s="12" t="str"/>
-      <c r="F301" s="14" t="str"/>
+      <c r="E301" s="14" t="str"/>
+      <c r="F301" s="12" t="str"/>
       <c r="G301" s="15" t="str"/>
     </row>
     <row r="302">
@@ -3149,8 +3149,8 @@
       <c r="B302" s="12" t="str"/>
       <c r="C302" s="13" t="str"/>
       <c r="D302" s="12" t="str"/>
-      <c r="E302" s="12" t="str"/>
-      <c r="F302" s="14" t="str"/>
+      <c r="E302" s="14" t="str"/>
+      <c r="F302" s="12" t="str"/>
       <c r="G302" s="15" t="str"/>
     </row>
     <row r="303">
@@ -3158,8 +3158,8 @@
       <c r="B303" s="12" t="str"/>
       <c r="C303" s="13" t="str"/>
       <c r="D303" s="12" t="str"/>
-      <c r="E303" s="12" t="str"/>
-      <c r="F303" s="14" t="str"/>
+      <c r="E303" s="14" t="str"/>
+      <c r="F303" s="12" t="str"/>
       <c r="G303" s="15" t="str"/>
     </row>
     <row r="304">
@@ -3167,8 +3167,8 @@
       <c r="B304" s="12" t="str"/>
       <c r="C304" s="13" t="str"/>
       <c r="D304" s="12" t="str"/>
-      <c r="E304" s="12" t="str"/>
-      <c r="F304" s="14" t="str"/>
+      <c r="E304" s="14" t="str"/>
+      <c r="F304" s="12" t="str"/>
       <c r="G304" s="15" t="str"/>
     </row>
     <row r="305">
@@ -3176,8 +3176,8 @@
       <c r="B305" s="12" t="str"/>
       <c r="C305" s="13" t="str"/>
       <c r="D305" s="12" t="str"/>
-      <c r="E305" s="12" t="str"/>
-      <c r="F305" s="14" t="str"/>
+      <c r="E305" s="14" t="str"/>
+      <c r="F305" s="12" t="str"/>
       <c r="G305" s="15" t="str"/>
     </row>
     <row r="306">
@@ -3185,8 +3185,8 @@
       <c r="B306" s="12" t="str"/>
       <c r="C306" s="13" t="str"/>
       <c r="D306" s="12" t="str"/>
-      <c r="E306" s="12" t="str"/>
-      <c r="F306" s="14" t="str"/>
+      <c r="E306" s="14" t="str"/>
+      <c r="F306" s="12" t="str"/>
       <c r="G306" s="15" t="str"/>
     </row>
     <row r="307">
@@ -3194,8 +3194,8 @@
       <c r="B307" s="12" t="str"/>
       <c r="C307" s="13" t="str"/>
       <c r="D307" s="12" t="str"/>
-      <c r="E307" s="12" t="str"/>
-      <c r="F307" s="14" t="str"/>
+      <c r="E307" s="14" t="str"/>
+      <c r="F307" s="12" t="str"/>
       <c r="G307" s="15" t="str"/>
     </row>
     <row r="308">
@@ -3203,8 +3203,8 @@
       <c r="B308" s="12" t="str"/>
       <c r="C308" s="13" t="str"/>
       <c r="D308" s="12" t="str"/>
-      <c r="E308" s="12" t="str"/>
-      <c r="F308" s="14" t="str"/>
+      <c r="E308" s="14" t="str"/>
+      <c r="F308" s="12" t="str"/>
       <c r="G308" s="15" t="str"/>
     </row>
     <row r="309">
@@ -3212,8 +3212,8 @@
       <c r="B309" s="12" t="str"/>
       <c r="C309" s="13" t="str"/>
       <c r="D309" s="12" t="str"/>
-      <c r="E309" s="12" t="str"/>
-      <c r="F309" s="14" t="str"/>
+      <c r="E309" s="14" t="str"/>
+      <c r="F309" s="12" t="str"/>
       <c r="G309" s="15" t="str"/>
     </row>
     <row r="310">
@@ -3221,8 +3221,8 @@
       <c r="B310" s="12" t="str"/>
       <c r="C310" s="13" t="str"/>
       <c r="D310" s="12" t="str"/>
-      <c r="E310" s="12" t="str"/>
-      <c r="F310" s="14" t="str"/>
+      <c r="E310" s="14" t="str"/>
+      <c r="F310" s="12" t="str"/>
       <c r="G310" s="15" t="str"/>
     </row>
     <row r="311">
@@ -3230,8 +3230,8 @@
       <c r="B311" s="12" t="str"/>
       <c r="C311" s="13" t="str"/>
       <c r="D311" s="12" t="str"/>
-      <c r="E311" s="12" t="str"/>
-      <c r="F311" s="14" t="str"/>
+      <c r="E311" s="14" t="str"/>
+      <c r="F311" s="12" t="str"/>
       <c r="G311" s="15" t="str"/>
     </row>
     <row r="312">
@@ -3239,8 +3239,8 @@
       <c r="B312" s="12" t="str"/>
       <c r="C312" s="13" t="str"/>
       <c r="D312" s="12" t="str"/>
-      <c r="E312" s="12" t="str"/>
-      <c r="F312" s="14" t="str"/>
+      <c r="E312" s="14" t="str"/>
+      <c r="F312" s="12" t="str"/>
       <c r="G312" s="15" t="str"/>
     </row>
     <row r="313">
@@ -3248,8 +3248,8 @@
       <c r="B313" s="12" t="str"/>
       <c r="C313" s="13" t="str"/>
       <c r="D313" s="12" t="str"/>
-      <c r="E313" s="12" t="str"/>
-      <c r="F313" s="14" t="str"/>
+      <c r="E313" s="14" t="str"/>
+      <c r="F313" s="12" t="str"/>
       <c r="G313" s="15" t="str"/>
     </row>
     <row r="314">
@@ -3257,8 +3257,8 @@
       <c r="B314" s="12" t="str"/>
       <c r="C314" s="13" t="str"/>
       <c r="D314" s="12" t="str"/>
-      <c r="E314" s="12" t="str"/>
-      <c r="F314" s="14" t="str"/>
+      <c r="E314" s="14" t="str"/>
+      <c r="F314" s="12" t="str"/>
       <c r="G314" s="15" t="str"/>
     </row>
     <row r="315">
@@ -3266,8 +3266,8 @@
       <c r="B315" s="12" t="str"/>
       <c r="C315" s="13" t="str"/>
       <c r="D315" s="12" t="str"/>
-      <c r="E315" s="12" t="str"/>
-      <c r="F315" s="14" t="str"/>
+      <c r="E315" s="14" t="str"/>
+      <c r="F315" s="12" t="str"/>
       <c r="G315" s="15" t="str"/>
     </row>
     <row r="316">
@@ -3275,8 +3275,8 @@
       <c r="B316" s="12" t="str"/>
       <c r="C316" s="13" t="str"/>
       <c r="D316" s="12" t="str"/>
-      <c r="E316" s="12" t="str"/>
-      <c r="F316" s="14" t="str"/>
+      <c r="E316" s="14" t="str"/>
+      <c r="F316" s="12" t="str"/>
       <c r="G316" s="15" t="str"/>
     </row>
     <row r="317">
@@ -3284,8 +3284,8 @@
       <c r="B317" s="12" t="str"/>
       <c r="C317" s="13" t="str"/>
       <c r="D317" s="12" t="str"/>
-      <c r="E317" s="12" t="str"/>
-      <c r="F317" s="14" t="str"/>
+      <c r="E317" s="14" t="str"/>
+      <c r="F317" s="12" t="str"/>
       <c r="G317" s="15" t="str"/>
     </row>
     <row r="318">
@@ -3293,8 +3293,8 @@
       <c r="B318" s="12" t="str"/>
       <c r="C318" s="13" t="str"/>
       <c r="D318" s="12" t="str"/>
-      <c r="E318" s="12" t="str"/>
-      <c r="F318" s="14" t="str"/>
+      <c r="E318" s="14" t="str"/>
+      <c r="F318" s="12" t="str"/>
       <c r="G318" s="15" t="str"/>
     </row>
     <row r="319">
@@ -3302,8 +3302,8 @@
       <c r="B319" s="12" t="str"/>
       <c r="C319" s="13" t="str"/>
       <c r="D319" s="12" t="str"/>
-      <c r="E319" s="12" t="str"/>
-      <c r="F319" s="14" t="str"/>
+      <c r="E319" s="14" t="str"/>
+      <c r="F319" s="12" t="str"/>
       <c r="G319" s="15" t="str"/>
     </row>
     <row r="320">
@@ -3311,8 +3311,8 @@
       <c r="B320" s="12" t="str"/>
       <c r="C320" s="13" t="str"/>
       <c r="D320" s="12" t="str"/>
-      <c r="E320" s="12" t="str"/>
-      <c r="F320" s="14" t="str"/>
+      <c r="E320" s="14" t="str"/>
+      <c r="F320" s="12" t="str"/>
       <c r="G320" s="15" t="str"/>
     </row>
     <row r="321">
@@ -3320,8 +3320,8 @@
       <c r="B321" s="12" t="str"/>
       <c r="C321" s="13" t="str"/>
       <c r="D321" s="12" t="str"/>
-      <c r="E321" s="12" t="str"/>
-      <c r="F321" s="14" t="str"/>
+      <c r="E321" s="14" t="str"/>
+      <c r="F321" s="12" t="str"/>
       <c r="G321" s="15" t="str"/>
     </row>
     <row r="322">
@@ -3329,8 +3329,8 @@
       <c r="B322" s="12" t="str"/>
       <c r="C322" s="13" t="str"/>
       <c r="D322" s="12" t="str"/>
-      <c r="E322" s="12" t="str"/>
-      <c r="F322" s="14" t="str"/>
+      <c r="E322" s="14" t="str"/>
+      <c r="F322" s="12" t="str"/>
       <c r="G322" s="15" t="str"/>
     </row>
     <row r="323">
@@ -3338,8 +3338,8 @@
       <c r="B323" s="12" t="str"/>
       <c r="C323" s="13" t="str"/>
       <c r="D323" s="12" t="str"/>
-      <c r="E323" s="12" t="str"/>
-      <c r="F323" s="14" t="str"/>
+      <c r="E323" s="14" t="str"/>
+      <c r="F323" s="12" t="str"/>
       <c r="G323" s="15" t="str"/>
     </row>
     <row r="324">
@@ -3347,8 +3347,8 @@
       <c r="B324" s="12" t="str"/>
       <c r="C324" s="13" t="str"/>
       <c r="D324" s="12" t="str"/>
-      <c r="E324" s="12" t="str"/>
-      <c r="F324" s="14" t="str"/>
+      <c r="E324" s="14" t="str"/>
+      <c r="F324" s="12" t="str"/>
       <c r="G324" s="15" t="str"/>
     </row>
     <row r="325">
@@ -3356,8 +3356,8 @@
       <c r="B325" s="12" t="str"/>
       <c r="C325" s="13" t="str"/>
       <c r="D325" s="12" t="str"/>
-      <c r="E325" s="12" t="str"/>
-      <c r="F325" s="14" t="str"/>
+      <c r="E325" s="14" t="str"/>
+      <c r="F325" s="12" t="str"/>
       <c r="G325" s="15" t="str"/>
     </row>
     <row r="326">
@@ -3365,8 +3365,8 @@
       <c r="B326" s="12" t="str"/>
       <c r="C326" s="13" t="str"/>
       <c r="D326" s="12" t="str"/>
-      <c r="E326" s="12" t="str"/>
-      <c r="F326" s="14" t="str"/>
+      <c r="E326" s="14" t="str"/>
+      <c r="F326" s="12" t="str"/>
       <c r="G326" s="15" t="str"/>
     </row>
     <row r="327">
@@ -3374,8 +3374,8 @@
       <c r="B327" s="12" t="str"/>
       <c r="C327" s="13" t="str"/>
       <c r="D327" s="12" t="str"/>
-      <c r="E327" s="12" t="str"/>
-      <c r="F327" s="14" t="str"/>
+      <c r="E327" s="14" t="str"/>
+      <c r="F327" s="12" t="str"/>
       <c r="G327" s="15" t="str"/>
     </row>
     <row r="328">
@@ -3383,8 +3383,8 @@
       <c r="B328" s="12" t="str"/>
       <c r="C328" s="13" t="str"/>
       <c r="D328" s="12" t="str"/>
-      <c r="E328" s="12" t="str"/>
-      <c r="F328" s="14" t="str"/>
+      <c r="E328" s="14" t="str"/>
+      <c r="F328" s="12" t="str"/>
       <c r="G328" s="15" t="str"/>
     </row>
     <row r="329">
@@ -3392,8 +3392,8 @@
       <c r="B329" s="12" t="str"/>
       <c r="C329" s="13" t="str"/>
       <c r="D329" s="12" t="str"/>
-      <c r="E329" s="12" t="str"/>
-      <c r="F329" s="14" t="str"/>
+      <c r="E329" s="14" t="str"/>
+      <c r="F329" s="12" t="str"/>
       <c r="G329" s="15" t="str"/>
     </row>
     <row r="330">
@@ -3401,8 +3401,8 @@
       <c r="B330" s="12" t="str"/>
       <c r="C330" s="13" t="str"/>
       <c r="D330" s="12" t="str"/>
-      <c r="E330" s="12" t="str"/>
-      <c r="F330" s="14" t="str"/>
+      <c r="E330" s="14" t="str"/>
+      <c r="F330" s="12" t="str"/>
       <c r="G330" s="15" t="str"/>
     </row>
     <row r="331">
@@ -3410,8 +3410,8 @@
       <c r="B331" s="12" t="str"/>
       <c r="C331" s="13" t="str"/>
       <c r="D331" s="12" t="str"/>
-      <c r="E331" s="12" t="str"/>
-      <c r="F331" s="14" t="str"/>
+      <c r="E331" s="14" t="str"/>
+      <c r="F331" s="12" t="str"/>
       <c r="G331" s="15" t="str"/>
     </row>
     <row r="332">
@@ -3419,8 +3419,8 @@
       <c r="B332" s="12" t="str"/>
       <c r="C332" s="13" t="str"/>
       <c r="D332" s="12" t="str"/>
-      <c r="E332" s="12" t="str"/>
-      <c r="F332" s="14" t="str"/>
+      <c r="E332" s="14" t="str"/>
+      <c r="F332" s="12" t="str"/>
       <c r="G332" s="15" t="str"/>
     </row>
     <row r="333">
@@ -3428,8 +3428,8 @@
       <c r="B333" s="12" t="str"/>
       <c r="C333" s="13" t="str"/>
       <c r="D333" s="12" t="str"/>
-      <c r="E333" s="12" t="str"/>
-      <c r="F333" s="14" t="str"/>
+      <c r="E333" s="14" t="str"/>
+      <c r="F333" s="12" t="str"/>
       <c r="G333" s="15" t="str"/>
     </row>
     <row r="334">
@@ -3437,8 +3437,8 @@
       <c r="B334" s="12" t="str"/>
       <c r="C334" s="13" t="str"/>
       <c r="D334" s="12" t="str"/>
-      <c r="E334" s="12" t="str"/>
-      <c r="F334" s="14" t="str"/>
+      <c r="E334" s="14" t="str"/>
+      <c r="F334" s="12" t="str"/>
       <c r="G334" s="15" t="str"/>
     </row>
     <row r="335">
@@ -3446,8 +3446,8 @@
       <c r="B335" s="12" t="str"/>
       <c r="C335" s="13" t="str"/>
       <c r="D335" s="12" t="str"/>
-      <c r="E335" s="12" t="str"/>
-      <c r="F335" s="14" t="str"/>
+      <c r="E335" s="14" t="str"/>
+      <c r="F335" s="12" t="str"/>
       <c r="G335" s="15" t="str"/>
     </row>
     <row r="336">
@@ -3455,8 +3455,8 @@
       <c r="B336" s="12" t="str"/>
       <c r="C336" s="13" t="str"/>
       <c r="D336" s="12" t="str"/>
-      <c r="E336" s="12" t="str"/>
-      <c r="F336" s="14" t="str"/>
+      <c r="E336" s="14" t="str"/>
+      <c r="F336" s="12" t="str"/>
       <c r="G336" s="15" t="str"/>
     </row>
     <row r="337">
@@ -3464,8 +3464,8 @@
       <c r="B337" s="12" t="str"/>
       <c r="C337" s="13" t="str"/>
       <c r="D337" s="12" t="str"/>
-      <c r="E337" s="12" t="str"/>
-      <c r="F337" s="14" t="str"/>
+      <c r="E337" s="14" t="str"/>
+      <c r="F337" s="12" t="str"/>
       <c r="G337" s="15" t="str"/>
     </row>
     <row r="338">
@@ -3473,8 +3473,8 @@
       <c r="B338" s="12" t="str"/>
       <c r="C338" s="13" t="str"/>
       <c r="D338" s="12" t="str"/>
-      <c r="E338" s="12" t="str"/>
-      <c r="F338" s="14" t="str"/>
+      <c r="E338" s="14" t="str"/>
+      <c r="F338" s="12" t="str"/>
       <c r="G338" s="15" t="str"/>
     </row>
     <row r="339">
@@ -3482,8 +3482,8 @@
       <c r="B339" s="12" t="str"/>
       <c r="C339" s="13" t="str"/>
       <c r="D339" s="12" t="str"/>
-      <c r="E339" s="12" t="str"/>
-      <c r="F339" s="14" t="str"/>
+      <c r="E339" s="14" t="str"/>
+      <c r="F339" s="12" t="str"/>
       <c r="G339" s="15" t="str"/>
     </row>
     <row r="340">
@@ -3491,8 +3491,8 @@
       <c r="B340" s="12" t="str"/>
       <c r="C340" s="13" t="str"/>
       <c r="D340" s="12" t="str"/>
-      <c r="E340" s="12" t="str"/>
-      <c r="F340" s="14" t="str"/>
+      <c r="E340" s="14" t="str"/>
+      <c r="F340" s="12" t="str"/>
       <c r="G340" s="15" t="str"/>
     </row>
     <row r="341">
@@ -3500,8 +3500,8 @@
       <c r="B341" s="12" t="str"/>
       <c r="C341" s="13" t="str"/>
       <c r="D341" s="12" t="str"/>
-      <c r="E341" s="12" t="str"/>
-      <c r="F341" s="14" t="str"/>
+      <c r="E341" s="14" t="str"/>
+      <c r="F341" s="12" t="str"/>
       <c r="G341" s="15" t="str"/>
     </row>
     <row r="342">
@@ -3509,8 +3509,8 @@
       <c r="B342" s="12" t="str"/>
       <c r="C342" s="13" t="str"/>
       <c r="D342" s="12" t="str"/>
-      <c r="E342" s="12" t="str"/>
-      <c r="F342" s="14" t="str"/>
+      <c r="E342" s="14" t="str"/>
+      <c r="F342" s="12" t="str"/>
       <c r="G342" s="15" t="str"/>
     </row>
     <row r="343">
@@ -3518,8 +3518,8 @@
       <c r="B343" s="12" t="str"/>
       <c r="C343" s="13" t="str"/>
       <c r="D343" s="12" t="str"/>
-      <c r="E343" s="12" t="str"/>
-      <c r="F343" s="14" t="str"/>
+      <c r="E343" s="14" t="str"/>
+      <c r="F343" s="12" t="str"/>
       <c r="G343" s="15" t="str"/>
     </row>
     <row r="344">
@@ -3527,8 +3527,8 @@
       <c r="B344" s="12" t="str"/>
       <c r="C344" s="13" t="str"/>
       <c r="D344" s="12" t="str"/>
-      <c r="E344" s="12" t="str"/>
-      <c r="F344" s="14" t="str"/>
+      <c r="E344" s="14" t="str"/>
+      <c r="F344" s="12" t="str"/>
       <c r="G344" s="15" t="str"/>
     </row>
     <row r="345">
@@ -3536,8 +3536,8 @@
       <c r="B345" s="12" t="str"/>
       <c r="C345" s="13" t="str"/>
       <c r="D345" s="12" t="str"/>
-      <c r="E345" s="12" t="str"/>
-      <c r="F345" s="14" t="str"/>
+      <c r="E345" s="14" t="str"/>
+      <c r="F345" s="12" t="str"/>
       <c r="G345" s="15" t="str"/>
     </row>
     <row r="346">
@@ -3545,8 +3545,8 @@
       <c r="B346" s="12" t="str"/>
       <c r="C346" s="13" t="str"/>
       <c r="D346" s="12" t="str"/>
-      <c r="E346" s="12" t="str"/>
-      <c r="F346" s="14" t="str"/>
+      <c r="E346" s="14" t="str"/>
+      <c r="F346" s="12" t="str"/>
       <c r="G346" s="15" t="str"/>
     </row>
     <row r="347">
@@ -3554,8 +3554,8 @@
       <c r="B347" s="12" t="str"/>
       <c r="C347" s="13" t="str"/>
       <c r="D347" s="12" t="str"/>
-      <c r="E347" s="12" t="str"/>
-      <c r="F347" s="14" t="str"/>
+      <c r="E347" s="14" t="str"/>
+      <c r="F347" s="12" t="str"/>
       <c r="G347" s="15" t="str"/>
     </row>
     <row r="348">
@@ -3563,8 +3563,8 @@
       <c r="B348" s="12" t="str"/>
       <c r="C348" s="13" t="str"/>
       <c r="D348" s="12" t="str"/>
-      <c r="E348" s="12" t="str"/>
-      <c r="F348" s="14" t="str"/>
+      <c r="E348" s="14" t="str"/>
+      <c r="F348" s="12" t="str"/>
       <c r="G348" s="15" t="str"/>
     </row>
     <row r="349">
@@ -3572,8 +3572,8 @@
       <c r="B349" s="12" t="str"/>
       <c r="C349" s="13" t="str"/>
       <c r="D349" s="12" t="str"/>
-      <c r="E349" s="12" t="str"/>
-      <c r="F349" s="14" t="str"/>
+      <c r="E349" s="14" t="str"/>
+      <c r="F349" s="12" t="str"/>
       <c r="G349" s="15" t="str"/>
     </row>
     <row r="350">
@@ -3581,8 +3581,8 @@
       <c r="B350" s="12" t="str"/>
       <c r="C350" s="13" t="str"/>
       <c r="D350" s="12" t="str"/>
-      <c r="E350" s="12" t="str"/>
-      <c r="F350" s="14" t="str"/>
+      <c r="E350" s="14" t="str"/>
+      <c r="F350" s="12" t="str"/>
       <c r="G350" s="15" t="str"/>
     </row>
     <row r="351">
@@ -3590,8 +3590,8 @@
       <c r="B351" s="12" t="str"/>
       <c r="C351" s="13" t="str"/>
       <c r="D351" s="12" t="str"/>
-      <c r="E351" s="12" t="str"/>
-      <c r="F351" s="14" t="str"/>
+      <c r="E351" s="14" t="str"/>
+      <c r="F351" s="12" t="str"/>
       <c r="G351" s="15" t="str"/>
     </row>
     <row r="352">
@@ -3599,8 +3599,8 @@
       <c r="B352" s="12" t="str"/>
       <c r="C352" s="13" t="str"/>
       <c r="D352" s="12" t="str"/>
-      <c r="E352" s="12" t="str"/>
-      <c r="F352" s="14" t="str"/>
+      <c r="E352" s="14" t="str"/>
+      <c r="F352" s="12" t="str"/>
       <c r="G352" s="15" t="str"/>
     </row>
     <row r="353">
@@ -3608,8 +3608,8 @@
       <c r="B353" s="12" t="str"/>
       <c r="C353" s="13" t="str"/>
       <c r="D353" s="12" t="str"/>
-      <c r="E353" s="12" t="str"/>
-      <c r="F353" s="14" t="str"/>
+      <c r="E353" s="14" t="str"/>
+      <c r="F353" s="12" t="str"/>
       <c r="G353" s="15" t="str"/>
     </row>
     <row r="354">
@@ -3617,8 +3617,8 @@
       <c r="B354" s="12" t="str"/>
       <c r="C354" s="13" t="str"/>
       <c r="D354" s="12" t="str"/>
-      <c r="E354" s="12" t="str"/>
-      <c r="F354" s="14" t="str"/>
+      <c r="E354" s="14" t="str"/>
+      <c r="F354" s="12" t="str"/>
       <c r="G354" s="15" t="str"/>
     </row>
     <row r="355">
@@ -3626,8 +3626,8 @@
       <c r="B355" s="12" t="str"/>
       <c r="C355" s="13" t="str"/>
       <c r="D355" s="12" t="str"/>
-      <c r="E355" s="12" t="str"/>
-      <c r="F355" s="14" t="str"/>
+      <c r="E355" s="14" t="str"/>
+      <c r="F355" s="12" t="str"/>
       <c r="G355" s="15" t="str"/>
     </row>
     <row r="356">
@@ -3635,8 +3635,8 @@
       <c r="B356" s="12" t="str"/>
       <c r="C356" s="13" t="str"/>
       <c r="D356" s="12" t="str"/>
-      <c r="E356" s="12" t="str"/>
-      <c r="F356" s="14" t="str"/>
+      <c r="E356" s="14" t="str"/>
+      <c r="F356" s="12" t="str"/>
       <c r="G356" s="15" t="str"/>
     </row>
     <row r="357">
@@ -3644,8 +3644,8 @@
       <c r="B357" s="12" t="str"/>
       <c r="C357" s="13" t="str"/>
       <c r="D357" s="12" t="str"/>
-      <c r="E357" s="12" t="str"/>
-      <c r="F357" s="14" t="str"/>
+      <c r="E357" s="14" t="str"/>
+      <c r="F357" s="12" t="str"/>
       <c r="G357" s="15" t="str"/>
     </row>
     <row r="358">
@@ -3653,8 +3653,8 @@
       <c r="B358" s="12" t="str"/>
       <c r="C358" s="13" t="str"/>
       <c r="D358" s="12" t="str"/>
-      <c r="E358" s="12" t="str"/>
-      <c r="F358" s="14" t="str"/>
+      <c r="E358" s="14" t="str"/>
+      <c r="F358" s="12" t="str"/>
       <c r="G358" s="15" t="str"/>
     </row>
     <row r="359">
@@ -3662,8 +3662,8 @@
       <c r="B359" s="12" t="str"/>
       <c r="C359" s="13" t="str"/>
       <c r="D359" s="12" t="str"/>
-      <c r="E359" s="12" t="str"/>
-      <c r="F359" s="14" t="str"/>
+      <c r="E359" s="14" t="str"/>
+      <c r="F359" s="12" t="str"/>
       <c r="G359" s="15" t="str"/>
     </row>
     <row r="360">
@@ -3671,8 +3671,8 @@
       <c r="B360" s="12" t="str"/>
       <c r="C360" s="13" t="str"/>
       <c r="D360" s="12" t="str"/>
-      <c r="E360" s="12" t="str"/>
-      <c r="F360" s="14" t="str"/>
+      <c r="E360" s="14" t="str"/>
+      <c r="F360" s="12" t="str"/>
       <c r="G360" s="15" t="str"/>
     </row>
     <row r="361">
@@ -3680,8 +3680,8 @@
       <c r="B361" s="12" t="str"/>
       <c r="C361" s="13" t="str"/>
       <c r="D361" s="12" t="str"/>
-      <c r="E361" s="12" t="str"/>
-      <c r="F361" s="14" t="str"/>
+      <c r="E361" s="14" t="str"/>
+      <c r="F361" s="12" t="str"/>
       <c r="G361" s="15" t="str"/>
     </row>
     <row r="362">
@@ -3689,8 +3689,8 @@
       <c r="B362" s="12" t="str"/>
       <c r="C362" s="13" t="str"/>
       <c r="D362" s="12" t="str"/>
-      <c r="E362" s="12" t="str"/>
-      <c r="F362" s="14" t="str"/>
+      <c r="E362" s="14" t="str"/>
+      <c r="F362" s="12" t="str"/>
       <c r="G362" s="15" t="str"/>
     </row>
     <row r="363">
@@ -3698,8 +3698,8 @@
       <c r="B363" s="12" t="str"/>
       <c r="C363" s="13" t="str"/>
       <c r="D363" s="12" t="str"/>
-      <c r="E363" s="12" t="str"/>
-      <c r="F363" s="14" t="str"/>
+      <c r="E363" s="14" t="str"/>
+      <c r="F363" s="12" t="str"/>
       <c r="G363" s="15" t="str"/>
     </row>
     <row r="364">
@@ -3707,8 +3707,8 @@
       <c r="B364" s="12" t="str"/>
       <c r="C364" s="13" t="str"/>
       <c r="D364" s="12" t="str"/>
-      <c r="E364" s="12" t="str"/>
-      <c r="F364" s="14" t="str"/>
+      <c r="E364" s="14" t="str"/>
+      <c r="F364" s="12" t="str"/>
       <c r="G364" s="15" t="str"/>
     </row>
     <row r="365">
@@ -3716,8 +3716,8 @@
       <c r="B365" s="12" t="str"/>
       <c r="C365" s="13" t="str"/>
       <c r="D365" s="12" t="str"/>
-      <c r="E365" s="12" t="str"/>
-      <c r="F365" s="14" t="str"/>
+      <c r="E365" s="14" t="str"/>
+      <c r="F365" s="12" t="str"/>
       <c r="G365" s="15" t="str"/>
     </row>
     <row r="366">
@@ -3725,8 +3725,8 @@
       <c r="B366" s="12" t="str"/>
       <c r="C366" s="13" t="str"/>
       <c r="D366" s="12" t="str"/>
-      <c r="E366" s="12" t="str"/>
-      <c r="F366" s="14" t="str"/>
+      <c r="E366" s="14" t="str"/>
+      <c r="F366" s="12" t="str"/>
       <c r="G366" s="15" t="str"/>
     </row>
     <row r="367">
@@ -3734,8 +3734,8 @@
       <c r="B367" s="12" t="str"/>
       <c r="C367" s="13" t="str"/>
       <c r="D367" s="12" t="str"/>
-      <c r="E367" s="12" t="str"/>
-      <c r="F367" s="14" t="str"/>
+      <c r="E367" s="14" t="str"/>
+      <c r="F367" s="12" t="str"/>
       <c r="G367" s="15" t="str"/>
     </row>
     <row r="368">
@@ -3743,8 +3743,8 @@
       <c r="B368" s="12" t="str"/>
       <c r="C368" s="13" t="str"/>
       <c r="D368" s="12" t="str"/>
-      <c r="E368" s="12" t="str"/>
-      <c r="F368" s="14" t="str"/>
+      <c r="E368" s="14" t="str"/>
+      <c r="F368" s="12" t="str"/>
       <c r="G368" s="15" t="str"/>
     </row>
     <row r="369">
@@ -3752,8 +3752,8 @@
       <c r="B369" s="12" t="str"/>
       <c r="C369" s="13" t="str"/>
       <c r="D369" s="12" t="str"/>
-      <c r="E369" s="12" t="str"/>
-      <c r="F369" s="14" t="str"/>
+      <c r="E369" s="14" t="str"/>
+      <c r="F369" s="12" t="str"/>
       <c r="G369" s="15" t="str"/>
     </row>
     <row r="370">
@@ -3761,8 +3761,8 @@
       <c r="B370" s="12" t="str"/>
       <c r="C370" s="13" t="str"/>
       <c r="D370" s="12" t="str"/>
-      <c r="E370" s="12" t="str"/>
-      <c r="F370" s="14" t="str"/>
+      <c r="E370" s="14" t="str"/>
+      <c r="F370" s="12" t="str"/>
       <c r="G370" s="15" t="str"/>
     </row>
     <row r="371">
@@ -3770,8 +3770,8 @@
       <c r="B371" s="12" t="str"/>
       <c r="C371" s="13" t="str"/>
       <c r="D371" s="12" t="str"/>
-      <c r="E371" s="12" t="str"/>
-      <c r="F371" s="14" t="str"/>
+      <c r="E371" s="14" t="str"/>
+      <c r="F371" s="12" t="str"/>
       <c r="G371" s="15" t="str"/>
     </row>
     <row r="372">
@@ -3779,8 +3779,8 @@
       <c r="B372" s="12" t="str"/>
       <c r="C372" s="13" t="str"/>
       <c r="D372" s="12" t="str"/>
-      <c r="E372" s="12" t="str"/>
-      <c r="F372" s="14" t="str"/>
+      <c r="E372" s="14" t="str"/>
+      <c r="F372" s="12" t="str"/>
       <c r="G372" s="15" t="str"/>
     </row>
     <row r="373">
@@ -3788,8 +3788,8 @@
       <c r="B373" s="12" t="str"/>
       <c r="C373" s="13" t="str"/>
       <c r="D373" s="12" t="str"/>
-      <c r="E373" s="12" t="str"/>
-      <c r="F373" s="14" t="str"/>
+      <c r="E373" s="14" t="str"/>
+      <c r="F373" s="12" t="str"/>
       <c r="G373" s="15" t="str"/>
     </row>
     <row r="374">
@@ -3797,8 +3797,8 @@
       <c r="B374" s="12" t="str"/>
       <c r="C374" s="13" t="str"/>
       <c r="D374" s="12" t="str"/>
-      <c r="E374" s="12" t="str"/>
-      <c r="F374" s="14" t="str"/>
+      <c r="E374" s="14" t="str"/>
+      <c r="F374" s="12" t="str"/>
       <c r="G374" s="15" t="str"/>
     </row>
     <row r="375">
@@ -3806,8 +3806,8 @@
       <c r="B375" s="12" t="str"/>
       <c r="C375" s="13" t="str"/>
       <c r="D375" s="12" t="str"/>
-      <c r="E375" s="12" t="str"/>
-      <c r="F375" s="14" t="str"/>
+      <c r="E375" s="14" t="str"/>
+      <c r="F375" s="12" t="str"/>
       <c r="G375" s="15" t="str"/>
     </row>
     <row r="376">
@@ -3815,8 +3815,8 @@
       <c r="B376" s="12" t="str"/>
       <c r="C376" s="13" t="str"/>
       <c r="D376" s="12" t="str"/>
-      <c r="E376" s="12" t="str"/>
-      <c r="F376" s="14" t="str"/>
+      <c r="E376" s="14" t="str"/>
+      <c r="F376" s="12" t="str"/>
       <c r="G376" s="15" t="str"/>
     </row>
     <row r="377">
@@ -3824,8 +3824,8 @@
       <c r="B377" s="12" t="str"/>
       <c r="C377" s="13" t="str"/>
       <c r="D377" s="12" t="str"/>
-      <c r="E377" s="12" t="str"/>
-      <c r="F377" s="14" t="str"/>
+      <c r="E377" s="14" t="str"/>
+      <c r="F377" s="12" t="str"/>
       <c r="G377" s="15" t="str"/>
     </row>
     <row r="378">
@@ -3833,8 +3833,8 @@
       <c r="B378" s="12" t="str"/>
       <c r="C378" s="13" t="str"/>
       <c r="D378" s="12" t="str"/>
-      <c r="E378" s="12" t="str"/>
-      <c r="F378" s="14" t="str"/>
+      <c r="E378" s="14" t="str"/>
+      <c r="F378" s="12" t="str"/>
       <c r="G378" s="15" t="str"/>
     </row>
     <row r="379">
@@ -3842,8 +3842,8 @@
       <c r="B379" s="12" t="str"/>
       <c r="C379" s="13" t="str"/>
       <c r="D379" s="12" t="str"/>
-      <c r="E379" s="12" t="str"/>
-      <c r="F379" s="14" t="str"/>
+      <c r="E379" s="14" t="str"/>
+      <c r="F379" s="12" t="str"/>
       <c r="G379" s="15" t="str"/>
     </row>
     <row r="380">
@@ -3851,8 +3851,8 @@
       <c r="B380" s="12" t="str"/>
       <c r="C380" s="13" t="str"/>
       <c r="D380" s="12" t="str"/>
-      <c r="E380" s="12" t="str"/>
-      <c r="F380" s="14" t="str"/>
+      <c r="E380" s="14" t="str"/>
+      <c r="F380" s="12" t="str"/>
       <c r="G380" s="15" t="str"/>
     </row>
     <row r="381">
@@ -3860,8 +3860,8 @@
       <c r="B381" s="12" t="str"/>
       <c r="C381" s="13" t="str"/>
       <c r="D381" s="12" t="str"/>
-      <c r="E381" s="12" t="str"/>
-      <c r="F381" s="14" t="str"/>
+      <c r="E381" s="14" t="str"/>
+      <c r="F381" s="12" t="str"/>
       <c r="G381" s="15" t="str"/>
     </row>
     <row r="382">
@@ -3869,8 +3869,8 @@
       <c r="B382" s="12" t="str"/>
       <c r="C382" s="13" t="str"/>
       <c r="D382" s="12" t="str"/>
-      <c r="E382" s="12" t="str"/>
-      <c r="F382" s="14" t="str"/>
+      <c r="E382" s="14" t="str"/>
+      <c r="F382" s="12" t="str"/>
       <c r="G382" s="15" t="str"/>
     </row>
     <row r="383">
@@ -3878,8 +3878,8 @@
       <c r="B383" s="12" t="str"/>
       <c r="C383" s="13" t="str"/>
       <c r="D383" s="12" t="str"/>
-      <c r="E383" s="12" t="str"/>
-      <c r="F383" s="14" t="str"/>
+      <c r="E383" s="14" t="str"/>
+      <c r="F383" s="12" t="str"/>
       <c r="G383" s="15" t="str"/>
     </row>
     <row r="384">
@@ -3887,8 +3887,8 @@
       <c r="B384" s="12" t="str"/>
       <c r="C384" s="13" t="str"/>
       <c r="D384" s="12" t="str"/>
-      <c r="E384" s="12" t="str"/>
-      <c r="F384" s="14" t="str"/>
+      <c r="E384" s="14" t="str"/>
+      <c r="F384" s="12" t="str"/>
       <c r="G384" s="15" t="str"/>
     </row>
     <row r="385">
@@ -3896,8 +3896,8 @@
       <c r="B385" s="12" t="str"/>
       <c r="C385" s="13" t="str"/>
       <c r="D385" s="12" t="str"/>
-      <c r="E385" s="12" t="str"/>
-      <c r="F385" s="14" t="str"/>
+      <c r="E385" s="14" t="str"/>
+      <c r="F385" s="12" t="str"/>
       <c r="G385" s="15" t="str"/>
     </row>
     <row r="386">
@@ -3905,8 +3905,8 @@
       <c r="B386" s="12" t="str"/>
       <c r="C386" s="13" t="str"/>
       <c r="D386" s="12" t="str"/>
-      <c r="E386" s="12" t="str"/>
-      <c r="F386" s="14" t="str"/>
+      <c r="E386" s="14" t="str"/>
+      <c r="F386" s="12" t="str"/>
       <c r="G386" s="15" t="str"/>
     </row>
     <row r="387">
@@ -3914,8 +3914,8 @@
       <c r="B387" s="12" t="str"/>
       <c r="C387" s="13" t="str"/>
       <c r="D387" s="12" t="str"/>
-      <c r="E387" s="12" t="str"/>
-      <c r="F387" s="14" t="str"/>
+      <c r="E387" s="14" t="str"/>
+      <c r="F387" s="12" t="str"/>
       <c r="G387" s="15" t="str"/>
     </row>
     <row r="388">
@@ -3923,8 +3923,8 @@
       <c r="B388" s="12" t="str"/>
       <c r="C388" s="13" t="str"/>
       <c r="D388" s="12" t="str"/>
-      <c r="E388" s="12" t="str"/>
-      <c r="F388" s="14" t="str"/>
+      <c r="E388" s="14" t="str"/>
+      <c r="F388" s="12" t="str"/>
       <c r="G388" s="15" t="str"/>
     </row>
     <row r="389">
@@ -3932,8 +3932,8 @@
       <c r="B389" s="12" t="str"/>
       <c r="C389" s="13" t="str"/>
       <c r="D389" s="12" t="str"/>
-      <c r="E389" s="12" t="str"/>
-      <c r="F389" s="14" t="str"/>
+      <c r="E389" s="14" t="str"/>
+      <c r="F389" s="12" t="str"/>
       <c r="G389" s="15" t="str"/>
     </row>
     <row r="390">
@@ -3941,8 +3941,8 @@
       <c r="B390" s="12" t="str"/>
       <c r="C390" s="13" t="str"/>
       <c r="D390" s="12" t="str"/>
-      <c r="E390" s="12" t="str"/>
-      <c r="F390" s="14" t="str"/>
+      <c r="E390" s="14" t="str"/>
+      <c r="F390" s="12" t="str"/>
       <c r="G390" s="15" t="str"/>
     </row>
     <row r="391">
@@ -3950,8 +3950,8 @@
       <c r="B391" s="12" t="str"/>
       <c r="C391" s="13" t="str"/>
       <c r="D391" s="12" t="str"/>
-      <c r="E391" s="12" t="str"/>
-      <c r="F391" s="14" t="str"/>
+      <c r="E391" s="14" t="str"/>
+      <c r="F391" s="12" t="str"/>
       <c r="G391" s="15" t="str"/>
     </row>
     <row r="392">
@@ -3959,8 +3959,8 @@
       <c r="B392" s="12" t="str"/>
       <c r="C392" s="13" t="str"/>
       <c r="D392" s="12" t="str"/>
-      <c r="E392" s="12" t="str"/>
-      <c r="F392" s="14" t="str"/>
+      <c r="E392" s="14" t="str"/>
+      <c r="F392" s="12" t="str"/>
       <c r="G392" s="15" t="str"/>
     </row>
     <row r="393">
@@ -3968,8 +3968,8 @@
       <c r="B393" s="12" t="str"/>
       <c r="C393" s="13" t="str"/>
       <c r="D393" s="12" t="str"/>
-      <c r="E393" s="12" t="str"/>
-      <c r="F393" s="14" t="str"/>
+      <c r="E393" s="14" t="str"/>
+      <c r="F393" s="12" t="str"/>
       <c r="G393" s="15" t="str"/>
     </row>
     <row r="394">
@@ -3977,8 +3977,8 @@
       <c r="B394" s="12" t="str"/>
       <c r="C394" s="13" t="str"/>
       <c r="D394" s="12" t="str"/>
-      <c r="E394" s="12" t="str"/>
-      <c r="F394" s="14" t="str"/>
+      <c r="E394" s="14" t="str"/>
+      <c r="F394" s="12" t="str"/>
       <c r="G394" s="15" t="str"/>
     </row>
     <row r="395">
@@ -3986,8 +3986,8 @@
       <c r="B395" s="12" t="str"/>
       <c r="C395" s="13" t="str"/>
       <c r="D395" s="12" t="str"/>
-      <c r="E395" s="12" t="str"/>
-      <c r="F395" s="14" t="str"/>
+      <c r="E395" s="14" t="str"/>
+      <c r="F395" s="12" t="str"/>
       <c r="G395" s="15" t="str"/>
     </row>
     <row r="396">
@@ -3995,8 +3995,8 @@
       <c r="B396" s="12" t="str"/>
       <c r="C396" s="13" t="str"/>
       <c r="D396" s="12" t="str"/>
-      <c r="E396" s="12" t="str"/>
-      <c r="F396" s="14" t="str"/>
+      <c r="E396" s="14" t="str"/>
+      <c r="F396" s="12" t="str"/>
       <c r="G396" s="15" t="str"/>
     </row>
     <row r="397">
@@ -4004,8 +4004,8 @@
       <c r="B397" s="12" t="str"/>
       <c r="C397" s="13" t="str"/>
       <c r="D397" s="12" t="str"/>
-      <c r="E397" s="12" t="str"/>
-      <c r="F397" s="14" t="str"/>
+      <c r="E397" s="14" t="str"/>
+      <c r="F397" s="12" t="str"/>
       <c r="G397" s="15" t="str"/>
     </row>
     <row r="398">
@@ -4013,8 +4013,8 @@
       <c r="B398" s="12" t="str"/>
       <c r="C398" s="13" t="str"/>
       <c r="D398" s="12" t="str"/>
-      <c r="E398" s="12" t="str"/>
-      <c r="F398" s="14" t="str"/>
+      <c r="E398" s="14" t="str"/>
+      <c r="F398" s="12" t="str"/>
       <c r="G398" s="15" t="str"/>
     </row>
     <row r="399">
@@ -4022,8 +4022,8 @@
       <c r="B399" s="12" t="str"/>
       <c r="C399" s="13" t="str"/>
       <c r="D399" s="12" t="str"/>
-      <c r="E399" s="12" t="str"/>
-      <c r="F399" s="14" t="str"/>
+      <c r="E399" s="14" t="str"/>
+      <c r="F399" s="12" t="str"/>
       <c r="G399" s="15" t="str"/>
     </row>
     <row r="400">
@@ -4031,8 +4031,8 @@
       <c r="B400" s="12" t="str"/>
       <c r="C400" s="13" t="str"/>
       <c r="D400" s="12" t="str"/>
-      <c r="E400" s="12" t="str"/>
-      <c r="F400" s="14" t="str"/>
+      <c r="E400" s="14" t="str"/>
+      <c r="F400" s="12" t="str"/>
       <c r="G400" s="15" t="str"/>
     </row>
     <row r="401">
@@ -4040,18 +4040,18 @@
       <c r="B401" s="12" t="str"/>
       <c r="C401" s="13" t="str"/>
       <c r="D401" s="12" t="str"/>
-      <c r="E401" s="12" t="str"/>
-      <c r="F401" s="14" t="str"/>
+      <c r="E401" s="14" t="str"/>
+      <c r="F401" s="12" t="str"/>
       <c r="G401" s="15" t="str"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="8B32"/>
   <autoFilter ref="A1:G401"/>
   <dataValidations count="3">
-    <dataValidation sqref="E2:E401" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F2:F401" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"ÚNICA,T/U,XS,S,M,L,XL,XXL,S/M,M/L,L/XL"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F401" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="whole" operator="between">
+    <dataValidation sqref="E2:E401" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="whole" operator="between">
       <formula1>1</formula1>
       <formula2>9999</formula2>
     </dataValidation>

</xml_diff>